<commit_message>
updated compositional analysis code and supplementary materials
</commit_message>
<xml_diff>
--- a/Supplementary_materials/Supplementary_Material_0_Sample_Metadata.xlsx
+++ b/Supplementary_materials/Supplementary_Material_0_Sample_Metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofcambridgecloud-my.sharepoint.com/personal/ck645_cam_ac_uk/Documents/Documents/GitHub/Central_Asia_islamic_ceramics/Supplementary_materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="8_{CE5D8AA6-F506-4BAB-B27C-85A234378BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{401699A8-8FB5-46D9-94AB-F1707A53FEF5}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="8_{CE5D8AA6-F506-4BAB-B27C-85A234378BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3F0EA84-284F-45DF-B343-D7E3F2F0B000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="645" xr2:uid="{7522CCE5-926C-4BF2-9BCC-E4C499424BA0}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Comparative NAA sample Metadata'!$A$1:$S$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sample Metadata'!$A$1:$S$167</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sample Metadata'!$A$1:$T$167</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5201" uniqueCount="1381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5358" uniqueCount="1536">
   <si>
     <t>Analytical ID (ANID)</t>
   </si>
@@ -4435,6 +4435,471 @@
   <si>
     <t>Shad Malik, 2018, R-4, bulk (Ш – М 2018 Р – 4 Отвал)</t>
   </si>
+  <si>
+    <t>Paste Description</t>
+  </si>
+  <si>
+    <t>fine fabric with some small voids, small red and black inclusions, and some very small white inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small voids and a very few small white inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with very minimal pores or inclusions visible.</t>
+  </si>
+  <si>
+    <t>fine fabric with some elongated voids (variety of sizes) with some reddish and white inclusions</t>
+  </si>
+  <si>
+    <t>very fine fabric with just a few small white inclusions and small voids.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small voids and some small darkish grey inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric with minimal pores and a few small reddish inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small reddish inclusions and some very elongated voids.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small elongated voids and some very small dark inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric with some small elongated voids and a few reddish angular inclusions as well as some smaller dark colored inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric with a few elongated voids and some small white inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric with no real inclusions visible, and only a few small voids.</t>
+  </si>
+  <si>
+    <t>fine fabric with some elongated voids in a variety of sizes and some small reddish brown inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with some elongated voids, some small white inclusions and larger reddish inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small elongated voids, and some very small inclusions that are either dark brown or white.</t>
+  </si>
+  <si>
+    <t>fine fabric with minimal voids and some reddish inclusions, including one large round very red particle.</t>
+  </si>
+  <si>
+    <t>very fine with some small white and reddish inclusions, and some small voids.</t>
+  </si>
+  <si>
+    <t>very fine, some small brownish black inclusions - but it looks like it is irregularly included.</t>
+  </si>
+  <si>
+    <t>fine fabric with minimal voids, and some small white inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with some voids in a variety of sizes and some small white inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric, just some small voids visible.</t>
+  </si>
+  <si>
+    <t>fine fabric with sime small elongated voids, medium sized reddish angular inclusions, and a very very small white inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small voids but very minimal inclusions overall.</t>
+  </si>
+  <si>
+    <t>fine fabric with minimal voids but some large angular reddish brown inclusions. Some smaller white inclusions also present.</t>
+  </si>
+  <si>
+    <t>very fine fabric with very few pores and some small dark and reddish inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric with some small reddish pink and dark colored inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with small white inclusions and small/medium sized reddish angular inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric with some small elongated voids and some very small dark colored inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small voids and a few small light colored inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric with minimal voids or inclusions.</t>
+  </si>
+  <si>
+    <t>the fabric is fairly heterogeneous and the paste looks like it has a range of oxidation with yellower and pinker sections. Some inclusions and voids. Very strange.</t>
+  </si>
+  <si>
+    <t>very fine with very few small inclusions, both reddish ones and white ones.</t>
+  </si>
+  <si>
+    <t>very fine fabric with some small voids, reddish inclusions (medium sized) and white inclusions (small).</t>
+  </si>
+  <si>
+    <t>fine fabric with some elongated voids, some small white inclusions, and larger reddish pink angular inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric with more oxidation on the exterior. Very minimal voids or inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small reddish inclusions and small round dark inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with some voids in a variety of sizes and some very small white inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric with only some small voids visible in the fresh break.</t>
+  </si>
+  <si>
+    <t>very fine fabric with some small pores and some very small dark and white inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with minimal voids and inclusions. Some small dark inclusions are visible.</t>
+  </si>
+  <si>
+    <t>fine fabric with some large white inclusions(?) that are of irregular shape.</t>
+  </si>
+  <si>
+    <t>fairly heterogeneous fabric with small to very large white and grayish inclusions visible in the fresh break.</t>
+  </si>
+  <si>
+    <t>fine fabric with white inclusions in a variety of sizes, including large inclusions. Voids are very small.</t>
+  </si>
+  <si>
+    <t>Fine fabric with only some small white inclusions visible. Voids are very very small.</t>
+  </si>
+  <si>
+    <t>fine fabric with some voids and a few very small white inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small voids and small dark (reddish?) inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric with some small voids and some very small dark inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with minimal pores and some small dark inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small elongated voids and some medium sized reddish inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small elongated voids and light colored inclusions. Evidence that the ceramic was burned.</t>
+  </si>
+  <si>
+    <t>medium fine fabric with a fair amount of inclusions, predominatly white inclusions in a variety of sizes.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small voids and small to medium sized reddish inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric with very minimal inclusions and voids.</t>
+  </si>
+  <si>
+    <t>very fine fabric with minimal inclusions and voids. Only a few very small dark inclusions visible.</t>
+  </si>
+  <si>
+    <t>very fine fabric with minimal pores and only one largish orange inclusion visible on the fresh break.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small voids. No visible inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric with some small voids and a couple of angular reddish inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with small white inclusions, and one large blocky red inclusion visible in the break</t>
+  </si>
+  <si>
+    <t>fine fabric with elongated voids. Very sandy.</t>
+  </si>
+  <si>
+    <t>Fabric is very fine, no visible voids or inclusions.</t>
+  </si>
+  <si>
+    <t>Very fine fabric with some small voids and small dark reddish brown inclusions</t>
+  </si>
+  <si>
+    <t>Very fine fabric with some very small voids present and a few small reddish inclusions</t>
+  </si>
+  <si>
+    <t>very fine fabric with some very elongated voids, parallel to the surface and some small dark inclusions</t>
+  </si>
+  <si>
+    <t>Very fine fabric, just a few very small voids and some very small dark inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric, some elongated voids and a few light reddish brown inclusions.</t>
+  </si>
+  <si>
+    <t>Very coarse fabric with medium and large blocky inclusions and lots of medium sized voids that have an elongated appearance. Very distinctive.</t>
+  </si>
+  <si>
+    <t>very fine fabric with some elongated voids and a very few small reddish inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric with some elongated voids, small reddish inclusions, and one small white inclusions visible.</t>
+  </si>
+  <si>
+    <t>Very fine fabric just with some elongated voids in a variety of sizes.</t>
+  </si>
+  <si>
+    <t>fairly heterogeneous fabric with small voids, white inclusions in a variety of sizes, and some small darker inclusions</t>
+  </si>
+  <si>
+    <t>very fine with only a few small voids visible.</t>
+  </si>
+  <si>
+    <t>fine with some small white inclusions and larger pinkish red and brown inclusions</t>
+  </si>
+  <si>
+    <t>Fine fabric with some small white inclusions ans some larger reddish inclusions which are angular.</t>
+  </si>
+  <si>
+    <t>fine with some small voids and very small white inclusions</t>
+  </si>
+  <si>
+    <t>fine fabric with some small voids, some small reddish inclusions which are blocky, and some small dark inclusions</t>
+  </si>
+  <si>
+    <t>very fine fabric with only a few voids and small dark inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with a few voids in a range of sizes, some angular reddish inclusions (medium sized), brownish grey inclusions (small to medium sized) and very small dark colored inclusions.</t>
+  </si>
+  <si>
+    <t>very fine, some elongated voids and small white inclusions. One elongated red inclusions visible in the break</t>
+  </si>
+  <si>
+    <t>very fine fabric with some small voids and some blocky reddish pink voids.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small white inclusions and minimal voids.</t>
+  </si>
+  <si>
+    <t>fine fabric with some voids in a variety of shapes and  round white inclusions visible.</t>
+  </si>
+  <si>
+    <t>fine(ish) fabric with white inclusions in a variety of sizes. Very distinctive.</t>
+  </si>
+  <si>
+    <t>very fine and dense fabric. Some small elongated voids and one medium sized white inclusion visible in the fresh break.</t>
+  </si>
+  <si>
+    <t>fine fabric with some elongated voids, angular brown inclusions and small white inclusions.</t>
+  </si>
+  <si>
+    <t>very fine with some small voids and small reddish and brown inclusions</t>
+  </si>
+  <si>
+    <t>fine fabric with small voids and small black inclusions and small round white inclusions.</t>
+  </si>
+  <si>
+    <t>very, very fine fabric with no visible inclusions</t>
+  </si>
+  <si>
+    <t>fine fabric with a few small voids, and some very small white inclusions.</t>
+  </si>
+  <si>
+    <t>fine(ish) fabric with some brown and dark gray inclusions on the inteiror, small to medium in size.</t>
+  </si>
+  <si>
+    <t>very fine fabric, slightly more oxidized on the interior than the exterior. Some whiteish inclusions in a variety of sizes.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small white inclusions and a very few larger dark inclusions.</t>
+  </si>
+  <si>
+    <t>very fine with some small reddish inclusions and small voids.</t>
+  </si>
+  <si>
+    <t>fine fabric with some voids in a variety of sizes. The interior is darker than the exterior portion.</t>
+  </si>
+  <si>
+    <t>Fine fabric but there is a gradient in fabric color with a yellow color by the rim and redder color towards the base. Fabic is fine with some small voids.</t>
+  </si>
+  <si>
+    <t>fine although fairly heterogeneous with some white inclusions in a range of sizes and elongated voids.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small voids, white inclusions in a variety of sizes, and some darkish grey inclusions which are angular and medium in size.</t>
+  </si>
+  <si>
+    <t>very fine fabric with some elongated pores. Almost sandy in texture but not soft.</t>
+  </si>
+  <si>
+    <t>very fine with only some very small voids visible.</t>
+  </si>
+  <si>
+    <t>very fine fabric, some small elongated voids and very small black inclusions</t>
+  </si>
+  <si>
+    <t>fine fabric with minimal pores and some very small brown/black inclusions.</t>
+  </si>
+  <si>
+    <t>some small white inclusions and one large reddish.</t>
+  </si>
+  <si>
+    <t>very fine, only a very few small voids visible.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small voids and largish brown blocky inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small voids and small black/brown inclusions.</t>
+  </si>
+  <si>
+    <t>fine with some smallish brown inclusions and voids in a range of sizes</t>
+  </si>
+  <si>
+    <t>very fine with no visible inclusions, just some voids in a range of sizes.</t>
+  </si>
+  <si>
+    <t>very fine with some medium small pinkish brown blocky inclusions and very small dark brown/black inclusions</t>
+  </si>
+  <si>
+    <t>very fine fabric with some small elongated voids and small inclusions including very small micaceous ones.</t>
+  </si>
+  <si>
+    <t>Fine with some white angular inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small voids and white angular inclusions</t>
+  </si>
+  <si>
+    <t>very fine fabric with some some small brown/black inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric with some small voids, medium sized reddish brown inclusions, and very small white and micaceous inclusions.</t>
+  </si>
+  <si>
+    <t>very fine fabric with some very small inclusions (brown and micaceous) and small voids.</t>
+  </si>
+  <si>
+    <t>very fine with a few small elongated voids, small white inclusions, and reddish brown inclusions.</t>
+  </si>
+  <si>
+    <t>very fine and dense with some small white inclusions.</t>
+  </si>
+  <si>
+    <t>very fine with elongated voids and small white round inclusions</t>
+  </si>
+  <si>
+    <t>some small voids and small  sized reddish brown inclusions</t>
+  </si>
+  <si>
+    <t>very fine some small white inclusions</t>
+  </si>
+  <si>
+    <t>very fine with very elongated voids and small white round inclusions</t>
+  </si>
+  <si>
+    <t>very fine, minimal voids, some round white inclusions</t>
+  </si>
+  <si>
+    <t>very fine with some elongated voids</t>
+  </si>
+  <si>
+    <t>very fine with some small voids and small round white inclusions and pink inclusions (almost the same color as the fabric)</t>
+  </si>
+  <si>
+    <t>very fine with only some small voids.</t>
+  </si>
+  <si>
+    <t>very fine, some voids and small reddish brown inclusions</t>
+  </si>
+  <si>
+    <t>fine fabric, some largish elongated voids and small white inclusions</t>
+  </si>
+  <si>
+    <t>fine with some elongated voids and lots of small white inclusions, and some micaceous inclusions.</t>
+  </si>
+  <si>
+    <t>very fine, only some medium sized voids.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small to very large sized voids.</t>
+  </si>
+  <si>
+    <t>very fine with some small voids.</t>
+  </si>
+  <si>
+    <t>very fine with some small and medium sized elongated voids.</t>
+  </si>
+  <si>
+    <t>fine fabric with minimal voids and small white inclusions</t>
+  </si>
+  <si>
+    <t>very fine fabric, only some very small voids.</t>
+  </si>
+  <si>
+    <t>very fine with some elongated voids and some small reddish brown inclusions.</t>
+  </si>
+  <si>
+    <t>fine with a wide range of void sizes and some small white inclusions.</t>
+  </si>
+  <si>
+    <t>fine with some voids, and both small white inclusions and larger angular reddish brown inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with some elongated voids and small micaceous inclusions.</t>
+  </si>
+  <si>
+    <t>fine with angular reeddish brown inclusions and small white round inclusions</t>
+  </si>
+  <si>
+    <t>fine fabric, minimal voids but one large visible reddish brown inclusion and some smaller white round inclusions.</t>
+  </si>
+  <si>
+    <t>very fine, only some voids visible.</t>
+  </si>
+  <si>
+    <t>very fine, almost no voids and some small white inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric, minimal voids some small white inclusions</t>
+  </si>
+  <si>
+    <t>fine fabric, some small white inclusions and minimal voids visible.</t>
+  </si>
+  <si>
+    <t>very fine with some small voids</t>
+  </si>
+  <si>
+    <t>very fine</t>
+  </si>
+  <si>
+    <t>fine with some very small voids and small round white inclusions.</t>
+  </si>
+  <si>
+    <t>very fine with only some small voids visible.</t>
+  </si>
+  <si>
+    <t>very fine with some very elongated voids and small white inclusions.</t>
+  </si>
+  <si>
+    <t>fine with some small voids and lots of small white inclusions.</t>
+  </si>
+  <si>
+    <t>fine with some elongated voids and small white inclusions.</t>
+  </si>
+  <si>
+    <t>fine with some small voids, and some brown and reddish brown inclusions visible.</t>
+  </si>
+  <si>
+    <t>fine with some small white and black inclusions, includind a medium sized plately white one.</t>
+  </si>
+  <si>
+    <t>very fine fabric with some small white inclusions visible.</t>
+  </si>
+  <si>
+    <t>fine fabric with minial pores but lots of small and medium sized white round inclusions.</t>
+  </si>
+  <si>
+    <t>fine fabric with some small voids.</t>
+  </si>
 </sst>
 </file>
 
@@ -4444,7 +4909,7 @@
     <numFmt numFmtId="164" formatCode="0_);[Red]\(0\)"/>
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4541,6 +5006,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -4616,7 +5086,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4855,6 +5325,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -5173,8 +5646,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{647BE94F-31AC-4288-9847-0E65BAB2173D}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:W167"/>
+  <dimension ref="A1:X167"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.21875" style="4" customWidth="1"/>
@@ -5188,14 +5660,14 @@
     <col min="12" max="12" width="19.44140625" style="20" customWidth="1"/>
     <col min="13" max="15" width="25.109375" style="4" customWidth="1"/>
     <col min="16" max="16" width="58.6640625" style="4" customWidth="1"/>
-    <col min="17" max="17" width="25.109375" style="10" customWidth="1"/>
-    <col min="18" max="18" width="33.33203125" style="10" customWidth="1"/>
-    <col min="19" max="19" width="65.6640625" style="42" customWidth="1"/>
-    <col min="20" max="20" width="31.109375" style="41" customWidth="1"/>
-    <col min="21" max="16384" width="8.88671875" style="10"/>
+    <col min="17" max="18" width="25.109375" style="10" customWidth="1"/>
+    <col min="19" max="19" width="33.33203125" style="10" customWidth="1"/>
+    <col min="20" max="20" width="65.6640625" style="42" customWidth="1"/>
+    <col min="21" max="21" width="31.109375" style="41" customWidth="1"/>
+    <col min="22" max="16384" width="8.88671875" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="3" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" s="3" customFormat="1" ht="72" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>777</v>
       </c>
@@ -5248,16 +5720,19 @@
         <v>12</v>
       </c>
       <c r="R1" s="3" t="s">
+        <v>1381</v>
+      </c>
+      <c r="S1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="S1" s="58" t="s">
+      <c r="T1" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="T1" s="60" t="s">
+      <c r="U1" s="60" t="s">
         <v>1310</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>223</v>
       </c>
@@ -5305,17 +5780,20 @@
       <c r="Q2" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="R2" s="10" t="s">
+      <c r="R2" s="85" t="s">
+        <v>1382</v>
+      </c>
+      <c r="S2" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S2" s="59" t="s">
+      <c r="T2" s="59" t="s">
         <v>1274</v>
       </c>
-      <c r="T2" s="80" t="s">
+      <c r="U2" s="80" t="s">
         <v>1311</v>
       </c>
     </row>
-    <row r="3" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>226</v>
       </c>
@@ -5363,17 +5841,20 @@
       <c r="Q3" s="10" t="s">
         <v>215</v>
       </c>
-      <c r="R3" s="10" t="s">
+      <c r="R3" s="85" t="s">
+        <v>1383</v>
+      </c>
+      <c r="S3" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S3" s="59" t="s">
+      <c r="T3" s="59" t="s">
         <v>1274</v>
       </c>
-      <c r="T3" s="80" t="s">
+      <c r="U3" s="80" t="s">
         <v>1311</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>217</v>
       </c>
@@ -5421,17 +5902,20 @@
       <c r="Q4" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="R4" s="10" t="s">
+      <c r="R4" s="85" t="s">
+        <v>1384</v>
+      </c>
+      <c r="S4" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S4" s="59" t="s">
+      <c r="T4" s="59" t="s">
         <v>1274</v>
       </c>
-      <c r="T4" s="80" t="s">
+      <c r="U4" s="80" t="s">
         <v>1311</v>
       </c>
     </row>
-    <row r="5" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>38</v>
       </c>
@@ -5477,17 +5961,20 @@
       <c r="Q5" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="R5" s="10" t="s">
+      <c r="R5" s="85" t="s">
+        <v>1385</v>
+      </c>
+      <c r="S5" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S5" s="59" t="s">
+      <c r="T5" s="59" t="s">
         <v>1275</v>
       </c>
-      <c r="T5" s="80" t="s">
+      <c r="U5" s="80" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="6" spans="1:20" ht="45" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" ht="45" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>49</v>
       </c>
@@ -5533,17 +6020,20 @@
       <c r="Q6" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="R6" s="10" t="s">
+      <c r="R6" s="85" t="s">
+        <v>1386</v>
+      </c>
+      <c r="S6" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S6" s="59" t="s">
+      <c r="T6" s="59" t="s">
         <v>1276</v>
       </c>
-      <c r="T6" s="80" t="s">
+      <c r="U6" s="80" t="s">
         <v>1313</v>
       </c>
     </row>
-    <row r="7" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>63</v>
       </c>
@@ -5591,17 +6081,20 @@
       <c r="Q7" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="R7" s="10" t="s">
+      <c r="R7" s="85" t="s">
+        <v>1387</v>
+      </c>
+      <c r="S7" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S7" s="80" t="s">
+      <c r="T7" s="80" t="s">
         <v>1277</v>
       </c>
-      <c r="T7" s="80" t="s">
+      <c r="U7" s="80" t="s">
         <v>1314</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>52</v>
       </c>
@@ -5649,17 +6142,20 @@
       <c r="Q8" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="R8" s="10" t="s">
+      <c r="R8" s="85" t="s">
+        <v>1388</v>
+      </c>
+      <c r="S8" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S8" s="80" t="s">
+      <c r="T8" s="80" t="s">
         <v>1277</v>
       </c>
-      <c r="T8" s="80" t="s">
+      <c r="U8" s="80" t="s">
         <v>1314</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>59</v>
       </c>
@@ -5707,17 +6203,20 @@
       <c r="Q9" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R9" s="10" t="s">
+      <c r="R9" s="85" t="s">
+        <v>1389</v>
+      </c>
+      <c r="S9" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S9" s="80" t="s">
+      <c r="T9" s="80" t="s">
         <v>1277</v>
       </c>
-      <c r="T9" s="80" t="s">
+      <c r="U9" s="80" t="s">
         <v>1314</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>68</v>
       </c>
@@ -5765,17 +6264,20 @@
       <c r="Q10" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="R10" s="10" t="s">
+      <c r="R10" s="85" t="s">
+        <v>1390</v>
+      </c>
+      <c r="S10" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S10" s="80" t="s">
+      <c r="T10" s="80" t="s">
         <v>1278</v>
       </c>
-      <c r="T10" s="80" t="s">
+      <c r="U10" s="80" t="s">
         <v>1314</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>74</v>
       </c>
@@ -5823,17 +6325,20 @@
       <c r="Q11" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="R11" s="10" t="s">
+      <c r="R11" s="85" t="s">
+        <v>1391</v>
+      </c>
+      <c r="S11" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S11" s="80" t="s">
+      <c r="T11" s="80" t="s">
         <v>1278</v>
       </c>
-      <c r="T11" s="80" t="s">
+      <c r="U11" s="80" t="s">
         <v>1314</v>
       </c>
     </row>
-    <row r="12" spans="1:20" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>89</v>
       </c>
@@ -5881,17 +6386,20 @@
       <c r="Q12" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R12" s="10" t="s">
+      <c r="R12" s="85" t="s">
+        <v>1392</v>
+      </c>
+      <c r="S12" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S12" s="81" t="s">
+      <c r="T12" s="81" t="s">
         <v>1279</v>
       </c>
-      <c r="T12" s="80" t="s">
+      <c r="U12" s="80" t="s">
         <v>1315</v>
       </c>
     </row>
-    <row r="13" spans="1:20" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>79</v>
       </c>
@@ -5935,17 +6443,20 @@
       <c r="Q13" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="R13" s="10" t="s">
+      <c r="R13" s="85" t="s">
+        <v>1393</v>
+      </c>
+      <c r="S13" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S13" s="81" t="s">
+      <c r="T13" s="81" t="s">
         <v>1279</v>
       </c>
-      <c r="T13" s="80" t="s">
+      <c r="U13" s="80" t="s">
         <v>1315</v>
       </c>
     </row>
-    <row r="14" spans="1:20" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>85</v>
       </c>
@@ -5993,17 +6504,20 @@
       <c r="Q14" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="R14" s="10" t="s">
+      <c r="R14" s="85" t="s">
+        <v>1394</v>
+      </c>
+      <c r="S14" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S14" s="81" t="s">
+      <c r="T14" s="81" t="s">
         <v>1279</v>
       </c>
-      <c r="T14" s="80" t="s">
+      <c r="U14" s="80" t="s">
         <v>1315</v>
       </c>
     </row>
-    <row r="15" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>17</v>
       </c>
@@ -6051,17 +6565,20 @@
       <c r="Q15" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R15" s="10" t="s">
+      <c r="R15" s="85" t="s">
+        <v>1395</v>
+      </c>
+      <c r="S15" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S15" s="80" t="s">
+      <c r="T15" s="80" t="s">
         <v>1280</v>
       </c>
-      <c r="T15" s="76" t="s">
+      <c r="U15" s="76" t="s">
         <v>1316</v>
       </c>
     </row>
-    <row r="16" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>93</v>
       </c>
@@ -6109,17 +6626,20 @@
       <c r="Q16" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R16" s="10" t="s">
+      <c r="R16" s="85" t="s">
+        <v>1396</v>
+      </c>
+      <c r="S16" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S16" s="80" t="s">
+      <c r="T16" s="80" t="s">
         <v>1282</v>
       </c>
-      <c r="T16" s="80" t="s">
+      <c r="U16" s="80" t="s">
         <v>1311</v>
       </c>
     </row>
-    <row r="17" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>96</v>
       </c>
@@ -6169,17 +6689,20 @@
       <c r="Q17" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R17" s="10" t="s">
+      <c r="R17" s="85" t="s">
+        <v>1397</v>
+      </c>
+      <c r="S17" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S17" s="80" t="s">
+      <c r="T17" s="80" t="s">
         <v>1282</v>
       </c>
-      <c r="T17" s="80" t="s">
+      <c r="U17" s="80" t="s">
         <v>1311</v>
       </c>
     </row>
-    <row r="18" spans="1:20" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>102</v>
       </c>
@@ -6227,17 +6750,20 @@
       <c r="Q18" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R18" s="10" t="s">
+      <c r="R18" s="85" t="s">
+        <v>1398</v>
+      </c>
+      <c r="S18" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S18" s="80" t="s">
+      <c r="T18" s="80" t="s">
         <v>1281</v>
       </c>
-      <c r="T18" s="80" t="s">
+      <c r="U18" s="80" t="s">
         <v>1311</v>
       </c>
     </row>
-    <row r="19" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>105</v>
       </c>
@@ -6279,17 +6805,20 @@
       <c r="Q19" s="41" t="s">
         <v>57</v>
       </c>
-      <c r="R19" s="10" t="s">
+      <c r="R19" s="85" t="s">
+        <v>1399</v>
+      </c>
+      <c r="S19" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S19" s="80" t="s">
+      <c r="T19" s="80" t="s">
         <v>1358</v>
       </c>
-      <c r="T19" s="80" t="s">
+      <c r="U19" s="80" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>113</v>
       </c>
@@ -6337,17 +6866,20 @@
       <c r="Q20" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R20" s="10" t="s">
+      <c r="R20" s="85" t="s">
+        <v>1400</v>
+      </c>
+      <c r="S20" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S20" s="80" t="s">
+      <c r="T20" s="80" t="s">
         <v>1283</v>
       </c>
-      <c r="T20" s="80" t="s">
+      <c r="U20" s="80" t="s">
         <v>1317</v>
       </c>
     </row>
-    <row r="21" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>117</v>
       </c>
@@ -6395,17 +6927,20 @@
       <c r="Q21" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="R21" s="10" t="s">
+      <c r="R21" s="85" t="s">
+        <v>1401</v>
+      </c>
+      <c r="S21" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S21" s="80" t="s">
+      <c r="T21" s="80" t="s">
         <v>1283</v>
       </c>
-      <c r="T21" s="80" t="s">
+      <c r="U21" s="80" t="s">
         <v>1317</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>122</v>
       </c>
@@ -6447,17 +6982,20 @@
       <c r="Q22" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="R22" s="10" t="s">
+      <c r="R22" s="85" t="s">
+        <v>1402</v>
+      </c>
+      <c r="S22" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S22" s="80" t="s">
+      <c r="T22" s="80" t="s">
         <v>1284</v>
       </c>
-      <c r="T22" s="80" t="s">
+      <c r="U22" s="80" t="s">
         <v>1311</v>
       </c>
     </row>
-    <row r="23" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>128</v>
       </c>
@@ -6505,17 +7043,20 @@
       <c r="Q23" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="R23" s="10" t="s">
+      <c r="R23" s="85" t="s">
+        <v>1403</v>
+      </c>
+      <c r="S23" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S23" s="80" t="s">
+      <c r="T23" s="80" t="s">
         <v>1284</v>
       </c>
-      <c r="T23" s="80" t="s">
+      <c r="U23" s="80" t="s">
         <v>1311</v>
       </c>
     </row>
-    <row r="24" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>131</v>
       </c>
@@ -6559,17 +7100,20 @@
       <c r="Q24" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R24" s="10" t="s">
+      <c r="R24" s="85" t="s">
+        <v>1404</v>
+      </c>
+      <c r="S24" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S24" s="81" t="s">
+      <c r="T24" s="81" t="s">
         <v>1285</v>
       </c>
-      <c r="T24" s="80" t="s">
+      <c r="U24" s="80" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="25" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>136</v>
       </c>
@@ -6617,17 +7161,20 @@
       <c r="Q25" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R25" s="10" t="s">
+      <c r="R25" s="85" t="s">
+        <v>1405</v>
+      </c>
+      <c r="S25" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S25" s="81" t="s">
+      <c r="T25" s="81" t="s">
         <v>1286</v>
       </c>
-      <c r="T25" s="80" t="s">
+      <c r="U25" s="80" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="26" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>141</v>
       </c>
@@ -6675,17 +7222,20 @@
       <c r="Q26" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="R26" s="10" t="s">
+      <c r="R26" s="85" t="s">
+        <v>1406</v>
+      </c>
+      <c r="S26" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S26" s="80" t="s">
+      <c r="T26" s="80" t="s">
         <v>1287</v>
       </c>
-      <c r="T26" s="80" t="s">
+      <c r="U26" s="80" t="s">
         <v>1318</v>
       </c>
     </row>
-    <row r="27" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>146</v>
       </c>
@@ -6733,17 +7283,20 @@
       <c r="Q27" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R27" s="10" t="s">
+      <c r="R27" s="85" t="s">
+        <v>1407</v>
+      </c>
+      <c r="S27" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S27" s="80" t="s">
+      <c r="T27" s="80" t="s">
         <v>1287</v>
       </c>
-      <c r="T27" s="80" t="s">
+      <c r="U27" s="80" t="s">
         <v>1318</v>
       </c>
     </row>
-    <row r="28" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>153</v>
       </c>
@@ -6789,17 +7342,20 @@
       <c r="Q28" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="R28" s="10" t="s">
+      <c r="R28" s="85" t="s">
+        <v>1408</v>
+      </c>
+      <c r="S28" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S28" s="80" t="s">
+      <c r="T28" s="80" t="s">
         <v>1288</v>
       </c>
-      <c r="T28" s="80" t="s">
+      <c r="U28" s="80" t="s">
         <v>1318</v>
       </c>
     </row>
-    <row r="29" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>149</v>
       </c>
@@ -6847,17 +7403,20 @@
       <c r="Q29" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="R29" s="10" t="s">
+      <c r="R29" s="85" t="s">
+        <v>1409</v>
+      </c>
+      <c r="S29" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S29" s="80" t="s">
+      <c r="T29" s="80" t="s">
         <v>1288</v>
       </c>
-      <c r="T29" s="80" t="s">
+      <c r="U29" s="80" t="s">
         <v>1318</v>
       </c>
     </row>
-    <row r="30" spans="1:20" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>157</v>
       </c>
@@ -6905,17 +7464,20 @@
       <c r="Q30" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="R30" s="10" t="s">
+      <c r="R30" s="85" t="s">
+        <v>1410</v>
+      </c>
+      <c r="S30" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S30" s="80" t="s">
+      <c r="T30" s="80" t="s">
         <v>1289</v>
       </c>
-      <c r="T30" s="80" t="s">
+      <c r="U30" s="80" t="s">
         <v>1318</v>
       </c>
     </row>
-    <row r="31" spans="1:20" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>161</v>
       </c>
@@ -6965,17 +7527,20 @@
       <c r="Q31" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="R31" s="10" t="s">
+      <c r="R31" s="85" t="s">
+        <v>1411</v>
+      </c>
+      <c r="S31" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S31" s="80" t="s">
+      <c r="T31" s="80" t="s">
         <v>1289</v>
       </c>
-      <c r="T31" s="80" t="s">
+      <c r="U31" s="80" t="s">
         <v>1318</v>
       </c>
     </row>
-    <row r="32" spans="1:20" ht="72" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>164</v>
       </c>
@@ -7021,17 +7586,20 @@
       <c r="Q32" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R32" s="10" t="s">
+      <c r="R32" s="85" t="s">
+        <v>1412</v>
+      </c>
+      <c r="S32" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S32" s="80" t="s">
+      <c r="T32" s="80" t="s">
         <v>1289</v>
       </c>
-      <c r="T32" s="80" t="s">
+      <c r="U32" s="80" t="s">
         <v>1318</v>
       </c>
     </row>
-    <row r="33" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>31</v>
       </c>
@@ -7079,17 +7647,20 @@
       <c r="Q33" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="R33" s="10" t="s">
+      <c r="R33" s="85" t="s">
+        <v>1413</v>
+      </c>
+      <c r="S33" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S33" s="80" t="s">
+      <c r="T33" s="80" t="s">
         <v>1290</v>
       </c>
-      <c r="T33" s="80" t="s">
+      <c r="U33" s="80" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="34" spans="1:20" ht="102.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:21" ht="102.6" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>169</v>
       </c>
@@ -7137,17 +7708,20 @@
       <c r="Q34" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R34" s="10" t="s">
+      <c r="R34" s="85" t="s">
+        <v>1414</v>
+      </c>
+      <c r="S34" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S34" s="59" t="s">
+      <c r="T34" s="59" t="s">
         <v>1291</v>
       </c>
-      <c r="T34" s="82" t="s">
+      <c r="U34" s="82" t="s">
         <v>1314</v>
       </c>
     </row>
-    <row r="35" spans="1:20" ht="102.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:21" ht="102.6" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>172</v>
       </c>
@@ -7195,17 +7769,20 @@
       <c r="Q35" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="R35" s="10" t="s">
+      <c r="R35" s="85" t="s">
+        <v>1415</v>
+      </c>
+      <c r="S35" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S35" s="59" t="s">
+      <c r="T35" s="59" t="s">
         <v>1291</v>
       </c>
-      <c r="T35" s="82" t="s">
+      <c r="U35" s="82" t="s">
         <v>1314</v>
       </c>
     </row>
-    <row r="36" spans="1:20" ht="102.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:21" ht="102.6" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>176</v>
       </c>
@@ -7255,17 +7832,20 @@
       <c r="Q36" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R36" s="10" t="s">
+      <c r="R36" s="85" t="s">
+        <v>1416</v>
+      </c>
+      <c r="S36" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S36" s="59" t="s">
+      <c r="T36" s="59" t="s">
         <v>1291</v>
       </c>
-      <c r="T36" s="82" t="s">
+      <c r="U36" s="82" t="s">
         <v>1314</v>
       </c>
     </row>
-    <row r="37" spans="1:20" ht="102.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:21" ht="102.6" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>179</v>
       </c>
@@ -7315,17 +7895,20 @@
       <c r="Q37" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R37" s="10" t="s">
+      <c r="R37" s="85" t="s">
+        <v>1417</v>
+      </c>
+      <c r="S37" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S37" s="59" t="s">
+      <c r="T37" s="59" t="s">
         <v>1291</v>
       </c>
-      <c r="T37" s="82" t="s">
+      <c r="U37" s="82" t="s">
         <v>1314</v>
       </c>
     </row>
-    <row r="38" spans="1:20" ht="102.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:21" ht="102.6" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
         <v>182</v>
       </c>
@@ -7367,17 +7950,20 @@
       <c r="Q38" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="R38" s="10" t="s">
+      <c r="R38" s="85" t="s">
+        <v>1418</v>
+      </c>
+      <c r="S38" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S38" s="59" t="s">
+      <c r="T38" s="59" t="s">
         <v>1291</v>
       </c>
-      <c r="T38" s="82" t="s">
+      <c r="U38" s="82" t="s">
         <v>1314</v>
       </c>
     </row>
-    <row r="39" spans="1:20" ht="102.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:21" ht="102.6" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>187</v>
       </c>
@@ -7425,17 +8011,20 @@
       <c r="Q39" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R39" s="10" t="s">
+      <c r="R39" s="85" t="s">
+        <v>1419</v>
+      </c>
+      <c r="S39" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S39" s="59" t="s">
+      <c r="T39" s="59" t="s">
         <v>1291</v>
       </c>
-      <c r="T39" s="82" t="s">
+      <c r="U39" s="82" t="s">
         <v>1314</v>
       </c>
     </row>
-    <row r="40" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>191</v>
       </c>
@@ -7483,17 +8072,20 @@
       <c r="Q40" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R40" s="10" t="s">
+      <c r="R40" s="85" t="s">
+        <v>1420</v>
+      </c>
+      <c r="S40" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S40" s="80" t="s">
+      <c r="T40" s="80" t="s">
         <v>1292</v>
       </c>
-      <c r="T40" s="82" t="s">
+      <c r="U40" s="82" t="s">
         <v>1317</v>
       </c>
     </row>
-    <row r="41" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>194</v>
       </c>
@@ -7541,17 +8133,20 @@
       <c r="Q41" s="41" t="s">
         <v>197</v>
       </c>
-      <c r="R41" s="10" t="s">
+      <c r="R41" s="85" t="s">
+        <v>1421</v>
+      </c>
+      <c r="S41" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S41" s="80" t="s">
+      <c r="T41" s="80" t="s">
         <v>1292</v>
       </c>
-      <c r="T41" s="82" t="s">
+      <c r="U41" s="82" t="s">
         <v>1317</v>
       </c>
     </row>
-    <row r="42" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>789</v>
       </c>
@@ -7599,17 +8194,20 @@
       <c r="Q42" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="R42" s="5" t="s">
+      <c r="R42" s="85" t="s">
+        <v>1422</v>
+      </c>
+      <c r="S42" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="S42" s="80" t="s">
+      <c r="T42" s="80" t="s">
         <v>1293</v>
       </c>
-      <c r="T42" s="82" t="s">
+      <c r="U42" s="82" t="s">
         <v>1317</v>
       </c>
     </row>
-    <row r="43" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
         <v>199</v>
       </c>
@@ -7657,17 +8255,20 @@
       <c r="Q43" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R43" s="10" t="s">
+      <c r="R43" s="85" t="s">
+        <v>1423</v>
+      </c>
+      <c r="S43" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S43" s="80" t="s">
+      <c r="T43" s="80" t="s">
         <v>1293</v>
       </c>
-      <c r="T43" s="82" t="s">
+      <c r="U43" s="82" t="s">
         <v>1317</v>
       </c>
     </row>
-    <row r="44" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>205</v>
       </c>
@@ -7715,17 +8316,20 @@
       <c r="Q44" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="R44" s="10" t="s">
+      <c r="R44" s="85" t="s">
+        <v>1424</v>
+      </c>
+      <c r="S44" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S44" s="80" t="s">
+      <c r="T44" s="80" t="s">
         <v>1294</v>
       </c>
-      <c r="T44" s="82" t="s">
+      <c r="U44" s="82" t="s">
         <v>1317</v>
       </c>
     </row>
-    <row r="45" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
         <v>213</v>
       </c>
@@ -7773,17 +8377,20 @@
       <c r="Q45" s="10" t="s">
         <v>215</v>
       </c>
-      <c r="R45" s="10" t="s">
+      <c r="R45" s="85" t="s">
+        <v>1425</v>
+      </c>
+      <c r="S45" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S45" s="81" t="s">
+      <c r="T45" s="81" t="s">
         <v>1295</v>
       </c>
-      <c r="T45" s="82" t="s">
+      <c r="U45" s="82" t="s">
         <v>1317</v>
       </c>
     </row>
-    <row r="46" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
         <v>209</v>
       </c>
@@ -7833,17 +8440,20 @@
       <c r="Q46" s="41" t="s">
         <v>211</v>
       </c>
-      <c r="R46" s="10" t="s">
+      <c r="R46" s="85" t="s">
+        <v>1426</v>
+      </c>
+      <c r="S46" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S46" s="81" t="s">
+      <c r="T46" s="81" t="s">
         <v>1295</v>
       </c>
-      <c r="T46" s="82" t="s">
+      <c r="U46" s="82" t="s">
         <v>1317</v>
       </c>
     </row>
-    <row r="47" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
         <v>230</v>
       </c>
@@ -7891,17 +8501,20 @@
       <c r="Q47" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="R47" s="10" t="s">
+      <c r="R47" s="85" t="s">
+        <v>1427</v>
+      </c>
+      <c r="S47" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S47" s="80" t="s">
+      <c r="T47" s="80" t="s">
         <v>1296</v>
       </c>
-      <c r="T47" s="82" t="s">
+      <c r="U47" s="82" t="s">
         <v>1319</v>
       </c>
     </row>
-    <row r="48" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
         <v>235</v>
       </c>
@@ -7949,17 +8562,20 @@
       <c r="Q48" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="R48" s="10" t="s">
+      <c r="R48" s="85" t="s">
+        <v>1428</v>
+      </c>
+      <c r="S48" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S48" s="80" t="s">
+      <c r="T48" s="80" t="s">
         <v>1297</v>
       </c>
-      <c r="T48" s="82" t="s">
+      <c r="U48" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="49" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>238</v>
       </c>
@@ -8009,17 +8625,20 @@
       <c r="Q49" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="R49" s="10" t="s">
+      <c r="R49" s="85" t="s">
+        <v>1429</v>
+      </c>
+      <c r="S49" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S49" s="80" t="s">
+      <c r="T49" s="80" t="s">
         <v>1297</v>
       </c>
-      <c r="T49" s="82" t="s">
+      <c r="U49" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="50" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
         <v>243</v>
       </c>
@@ -8067,17 +8686,20 @@
       <c r="Q50" s="41" t="s">
         <v>246</v>
       </c>
-      <c r="R50" s="10" t="s">
+      <c r="R50" s="85" t="s">
+        <v>1430</v>
+      </c>
+      <c r="S50" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S50" s="80" t="s">
+      <c r="T50" s="80" t="s">
         <v>1298</v>
       </c>
-      <c r="T50" s="82" t="s">
+      <c r="U50" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="51" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
         <v>248</v>
       </c>
@@ -8127,17 +8749,20 @@
       <c r="Q51" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="R51" s="10" t="s">
+      <c r="R51" s="85" t="s">
+        <v>1431</v>
+      </c>
+      <c r="S51" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S51" s="59" t="s">
+      <c r="T51" s="59" t="s">
         <v>1299</v>
       </c>
-      <c r="T51" s="82" t="s">
+      <c r="U51" s="82" t="s">
         <v>1320</v>
       </c>
     </row>
-    <row r="52" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
         <v>261</v>
       </c>
@@ -8187,17 +8812,20 @@
       <c r="Q52" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="R52" s="10" t="s">
+      <c r="R52" s="85" t="s">
+        <v>1432</v>
+      </c>
+      <c r="S52" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S52" s="59" t="s">
+      <c r="T52" s="59" t="s">
         <v>1299</v>
       </c>
-      <c r="T52" s="82" t="s">
+      <c r="U52" s="82" t="s">
         <v>1320</v>
       </c>
     </row>
-    <row r="53" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
         <v>251</v>
       </c>
@@ -8249,17 +8877,20 @@
       <c r="Q53" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R53" s="10" t="s">
+      <c r="R53" s="85" t="s">
+        <v>1433</v>
+      </c>
+      <c r="S53" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S53" s="59" t="s">
+      <c r="T53" s="59" t="s">
         <v>1299</v>
       </c>
-      <c r="T53" s="82" t="s">
+      <c r="U53" s="82" t="s">
         <v>1320</v>
       </c>
     </row>
-    <row r="54" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
         <v>268</v>
       </c>
@@ -8309,17 +8940,20 @@
       <c r="Q54" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="R54" s="10" t="s">
+      <c r="R54" s="85" t="s">
+        <v>1434</v>
+      </c>
+      <c r="S54" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S54" s="59" t="s">
+      <c r="T54" s="59" t="s">
         <v>1299</v>
       </c>
-      <c r="T54" s="82" t="s">
+      <c r="U54" s="82" t="s">
         <v>1320</v>
       </c>
     </row>
-    <row r="55" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A55" s="26" t="s">
         <v>793</v>
       </c>
@@ -8367,17 +9001,20 @@
       <c r="Q55" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="R55" s="5" t="s">
+      <c r="R55" s="85" t="s">
+        <v>1435</v>
+      </c>
+      <c r="S55" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="S55" s="59" t="s">
+      <c r="T55" s="59" t="s">
         <v>1299</v>
       </c>
-      <c r="T55" s="82" t="s">
+      <c r="U55" s="82" t="s">
         <v>1320</v>
       </c>
     </row>
-    <row r="56" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
         <v>274</v>
       </c>
@@ -8419,17 +9056,20 @@
       <c r="Q56" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="R56" s="10" t="s">
+      <c r="R56" s="85" t="s">
+        <v>1436</v>
+      </c>
+      <c r="S56" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S56" s="59" t="s">
+      <c r="T56" s="59" t="s">
         <v>1299</v>
       </c>
-      <c r="T56" s="82" t="s">
+      <c r="U56" s="82" t="s">
         <v>1320</v>
       </c>
     </row>
-    <row r="57" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
         <v>254</v>
       </c>
@@ -8477,17 +9117,20 @@
       <c r="Q57" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R57" s="10" t="s">
+      <c r="R57" s="85" t="s">
+        <v>1437</v>
+      </c>
+      <c r="S57" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S57" s="59" t="s">
+      <c r="T57" s="59" t="s">
         <v>1299</v>
       </c>
-      <c r="T57" s="82" t="s">
+      <c r="U57" s="82" t="s">
         <v>1320</v>
       </c>
     </row>
-    <row r="58" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
         <v>257</v>
       </c>
@@ -8537,17 +9180,20 @@
       <c r="Q58" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="R58" s="10" t="s">
+      <c r="R58" s="85" t="s">
+        <v>1438</v>
+      </c>
+      <c r="S58" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S58" s="59" t="s">
+      <c r="T58" s="59" t="s">
         <v>1299</v>
       </c>
-      <c r="T58" s="82" t="s">
+      <c r="U58" s="82" t="s">
         <v>1320</v>
       </c>
     </row>
-    <row r="59" spans="1:20" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
         <v>280</v>
       </c>
@@ -8589,17 +9235,20 @@
       <c r="Q59" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R59" s="10" t="s">
+      <c r="R59" s="85" t="s">
+        <v>1439</v>
+      </c>
+      <c r="S59" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S59" s="80" t="s">
+      <c r="T59" s="80" t="s">
         <v>1301</v>
       </c>
-      <c r="T59" s="82" t="s">
+      <c r="U59" s="82" t="s">
         <v>1321</v>
       </c>
     </row>
-    <row r="60" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A60" s="5" t="s">
         <v>283</v>
       </c>
@@ -8645,17 +9294,20 @@
       <c r="Q60" s="41" t="s">
         <v>57</v>
       </c>
-      <c r="R60" s="10" t="s">
+      <c r="R60" s="85" t="s">
+        <v>1440</v>
+      </c>
+      <c r="S60" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S60" s="80" t="s">
+      <c r="T60" s="80" t="s">
         <v>1301</v>
       </c>
-      <c r="T60" s="82" t="s">
+      <c r="U60" s="82" t="s">
         <v>1321</v>
       </c>
     </row>
-    <row r="61" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A61" s="26" t="s">
         <v>822</v>
       </c>
@@ -8701,17 +9353,20 @@
       <c r="Q61" s="33" t="s">
         <v>47</v>
       </c>
-      <c r="R61" s="5" t="s">
+      <c r="R61" s="85" t="s">
+        <v>1441</v>
+      </c>
+      <c r="S61" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="S61" s="83" t="s">
+      <c r="T61" s="83" t="s">
         <v>1361</v>
       </c>
-      <c r="T61" s="82" t="s">
+      <c r="U61" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="62" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
         <v>288</v>
       </c>
@@ -8761,17 +9416,20 @@
       <c r="Q62" s="41" t="s">
         <v>211</v>
       </c>
-      <c r="R62" s="10" t="s">
+      <c r="R62" s="85" t="s">
+        <v>1442</v>
+      </c>
+      <c r="S62" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S62" s="59" t="s">
+      <c r="T62" s="59" t="s">
         <v>1301</v>
       </c>
-      <c r="T62" s="82" t="s">
+      <c r="U62" s="82" t="s">
         <v>1321</v>
       </c>
     </row>
-    <row r="63" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
         <v>292</v>
       </c>
@@ -8819,17 +9477,20 @@
       <c r="Q63" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R63" s="10" t="s">
+      <c r="R63" s="85" t="s">
+        <v>1443</v>
+      </c>
+      <c r="S63" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S63" s="59" t="s">
+      <c r="T63" s="59" t="s">
         <v>1301</v>
       </c>
-      <c r="T63" s="82" t="s">
+      <c r="U63" s="82" t="s">
         <v>1321</v>
       </c>
     </row>
-    <row r="64" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
         <v>297</v>
       </c>
@@ -8877,17 +9538,20 @@
       <c r="Q64" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="R64" s="10" t="s">
+      <c r="R64" s="85" t="s">
+        <v>1444</v>
+      </c>
+      <c r="S64" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S64" s="59" t="s">
+      <c r="T64" s="59" t="s">
         <v>1301</v>
       </c>
-      <c r="T64" s="82" t="s">
+      <c r="U64" s="82" t="s">
         <v>1321</v>
       </c>
     </row>
-    <row r="65" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
         <v>300</v>
       </c>
@@ -8937,17 +9601,20 @@
       <c r="Q65" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R65" s="10" t="s">
+      <c r="R65" s="85" t="s">
+        <v>1445</v>
+      </c>
+      <c r="S65" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S65" s="59" t="s">
+      <c r="T65" s="59" t="s">
         <v>1301</v>
       </c>
-      <c r="T65" s="82" t="s">
+      <c r="U65" s="82" t="s">
         <v>1321</v>
       </c>
     </row>
-    <row r="66" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
         <v>303</v>
       </c>
@@ -8989,17 +9656,20 @@
       <c r="Q66" s="41" t="s">
         <v>57</v>
       </c>
-      <c r="R66" s="10" t="s">
+      <c r="R66" s="85" t="s">
+        <v>1446</v>
+      </c>
+      <c r="S66" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S66" s="80" t="s">
+      <c r="T66" s="80" t="s">
         <v>1303</v>
       </c>
-      <c r="T66" s="82" t="s">
+      <c r="U66" s="82" t="s">
         <v>1320</v>
       </c>
     </row>
-    <row r="67" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
         <v>306</v>
       </c>
@@ -9045,17 +9715,20 @@
       <c r="Q67" s="41" t="s">
         <v>308</v>
       </c>
-      <c r="R67" s="10" t="s">
+      <c r="R67" s="85" t="s">
+        <v>1447</v>
+      </c>
+      <c r="S67" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S67" s="80" t="s">
+      <c r="T67" s="80" t="s">
         <v>1303</v>
       </c>
-      <c r="T67" s="82" t="s">
+      <c r="U67" s="82" t="s">
         <v>1320</v>
       </c>
     </row>
-    <row r="68" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A68" s="5" t="s">
         <v>310</v>
       </c>
@@ -9097,17 +9770,20 @@
       <c r="Q68" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="R68" s="10" t="s">
+      <c r="R68" s="85" t="s">
+        <v>1448</v>
+      </c>
+      <c r="S68" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S68" s="80" t="s">
+      <c r="T68" s="80" t="s">
         <v>1303</v>
       </c>
-      <c r="T68" s="82" t="s">
+      <c r="U68" s="82" t="s">
         <v>1320</v>
       </c>
     </row>
-    <row r="69" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A69" s="5" t="s">
         <v>314</v>
       </c>
@@ -9155,17 +9831,20 @@
       <c r="Q69" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="R69" s="10" t="s">
+      <c r="R69" s="85" t="s">
+        <v>1449</v>
+      </c>
+      <c r="S69" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S69" s="80" t="s">
+      <c r="T69" s="80" t="s">
         <v>1303</v>
       </c>
-      <c r="T69" s="82" t="s">
+      <c r="U69" s="82" t="s">
         <v>1320</v>
       </c>
     </row>
-    <row r="70" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A70" s="5" t="s">
         <v>318</v>
       </c>
@@ -9207,17 +9886,20 @@
       <c r="Q70" s="10" t="s">
         <v>321</v>
       </c>
-      <c r="R70" s="10" t="s">
+      <c r="R70" s="85" t="s">
+        <v>1450</v>
+      </c>
+      <c r="S70" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S70" s="80" t="s">
+      <c r="T70" s="80" t="s">
         <v>1303</v>
       </c>
-      <c r="T70" s="82" t="s">
+      <c r="U70" s="82" t="s">
         <v>1320</v>
       </c>
     </row>
-    <row r="71" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
         <v>323</v>
       </c>
@@ -9265,17 +9947,20 @@
       <c r="Q71" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="R71" s="10" t="s">
+      <c r="R71" s="85" t="s">
+        <v>1451</v>
+      </c>
+      <c r="S71" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S71" s="80" t="s">
+      <c r="T71" s="80" t="s">
         <v>1300</v>
       </c>
-      <c r="T71" s="82" t="s">
+      <c r="U71" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="72" spans="1:20" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A72" s="26" t="s">
         <v>780</v>
       </c>
@@ -9319,17 +10004,20 @@
       <c r="Q72" s="33" t="s">
         <v>783</v>
       </c>
-      <c r="R72" s="5" t="s">
+      <c r="R72" s="85" t="s">
+        <v>1452</v>
+      </c>
+      <c r="S72" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="S72" s="80" t="s">
+      <c r="T72" s="80" t="s">
         <v>1300</v>
       </c>
-      <c r="T72" s="82" t="s">
+      <c r="U72" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="73" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
         <v>330</v>
       </c>
@@ -9377,17 +10065,20 @@
       <c r="Q73" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R73" s="10" t="s">
+      <c r="R73" s="85" t="s">
+        <v>1453</v>
+      </c>
+      <c r="S73" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S73" s="80" t="s">
+      <c r="T73" s="80" t="s">
         <v>1359</v>
       </c>
-      <c r="T73" s="82" t="s">
+      <c r="U73" s="82" t="s">
         <v>1360</v>
       </c>
     </row>
-    <row r="74" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A74" s="5" t="s">
         <v>333</v>
       </c>
@@ -9435,17 +10126,20 @@
       <c r="Q74" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R74" s="10" t="s">
+      <c r="R74" s="85" t="s">
+        <v>1454</v>
+      </c>
+      <c r="S74" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S74" s="80" t="s">
+      <c r="T74" s="80" t="s">
         <v>1359</v>
       </c>
-      <c r="T74" s="82" t="s">
+      <c r="U74" s="82" t="s">
         <v>1360</v>
       </c>
     </row>
-    <row r="75" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
         <v>338</v>
       </c>
@@ -9493,17 +10187,20 @@
       <c r="Q75" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R75" s="10" t="s">
+      <c r="R75" s="85" t="s">
+        <v>1455</v>
+      </c>
+      <c r="S75" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S75" s="80" t="s">
+      <c r="T75" s="80" t="s">
         <v>1359</v>
       </c>
-      <c r="T75" s="82" t="s">
+      <c r="U75" s="82" t="s">
         <v>1360</v>
       </c>
     </row>
-    <row r="76" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A76" s="5" t="s">
         <v>342</v>
       </c>
@@ -9555,17 +10252,20 @@
       <c r="Q76" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R76" s="10" t="s">
+      <c r="R76" s="85" t="s">
+        <v>1456</v>
+      </c>
+      <c r="S76" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S76" s="80" t="s">
+      <c r="T76" s="80" t="s">
         <v>1359</v>
       </c>
-      <c r="T76" s="82" t="s">
+      <c r="U76" s="82" t="s">
         <v>1360</v>
       </c>
     </row>
-    <row r="77" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
         <v>346</v>
       </c>
@@ -9615,17 +10315,20 @@
       <c r="Q77" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="R77" s="10" t="s">
+      <c r="R77" s="85" t="s">
+        <v>1457</v>
+      </c>
+      <c r="S77" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S77" s="80" t="s">
+      <c r="T77" s="80" t="s">
         <v>1359</v>
       </c>
-      <c r="T77" s="82" t="s">
+      <c r="U77" s="82" t="s">
         <v>1360</v>
       </c>
     </row>
-    <row r="78" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A78" s="5" t="s">
         <v>327</v>
       </c>
@@ -9673,17 +10376,20 @@
       <c r="Q78" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R78" s="10" t="s">
+      <c r="R78" s="85" t="s">
+        <v>1458</v>
+      </c>
+      <c r="S78" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S78" s="80" t="s">
+      <c r="T78" s="80" t="s">
         <v>1359</v>
       </c>
-      <c r="T78" s="82" t="s">
+      <c r="U78" s="82" t="s">
         <v>1360</v>
       </c>
     </row>
-    <row r="79" spans="1:20" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
         <v>350</v>
       </c>
@@ -9725,17 +10431,20 @@
       <c r="Q79" s="10" t="s">
         <v>352</v>
       </c>
-      <c r="R79" s="10" t="s">
+      <c r="R79" s="85" t="s">
+        <v>1459</v>
+      </c>
+      <c r="S79" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S79" s="80" t="s">
+      <c r="T79" s="80" t="s">
         <v>1359</v>
       </c>
-      <c r="T79" s="82" t="s">
+      <c r="U79" s="82" t="s">
         <v>1360</v>
       </c>
     </row>
-    <row r="80" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
         <v>354</v>
       </c>
@@ -9783,17 +10492,20 @@
       <c r="Q80" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R80" s="10" t="s">
+      <c r="R80" s="85" t="s">
+        <v>1460</v>
+      </c>
+      <c r="S80" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S80" s="80" t="s">
+      <c r="T80" s="80" t="s">
         <v>1359</v>
       </c>
-      <c r="T80" s="82" t="s">
+      <c r="U80" s="82" t="s">
         <v>1360</v>
       </c>
     </row>
-    <row r="81" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
         <v>357</v>
       </c>
@@ -9841,17 +10553,20 @@
       <c r="Q81" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R81" s="10" t="s">
+      <c r="R81" s="85" t="s">
+        <v>1461</v>
+      </c>
+      <c r="S81" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S81" s="80" t="s">
+      <c r="T81" s="80" t="s">
         <v>1359</v>
       </c>
-      <c r="T81" s="82" t="s">
+      <c r="U81" s="82" t="s">
         <v>1360</v>
       </c>
     </row>
-    <row r="82" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A82" s="5" t="s">
         <v>361</v>
       </c>
@@ -9899,17 +10614,20 @@
       <c r="Q82" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R82" s="10" t="s">
+      <c r="R82" s="85" t="s">
+        <v>1462</v>
+      </c>
+      <c r="S82" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S82" s="80" t="s">
+      <c r="T82" s="80" t="s">
         <v>1359</v>
       </c>
-      <c r="T82" s="82" t="s">
+      <c r="U82" s="82" t="s">
         <v>1360</v>
       </c>
     </row>
-    <row r="83" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A83" s="5" t="s">
         <v>365</v>
       </c>
@@ -9955,17 +10673,20 @@
       <c r="Q83" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="R83" s="10" t="s">
+      <c r="R83" s="85" t="s">
+        <v>1463</v>
+      </c>
+      <c r="S83" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S83" s="80" t="s">
+      <c r="T83" s="80" t="s">
         <v>1300</v>
       </c>
-      <c r="T83" s="82" t="s">
+      <c r="U83" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="84" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A84" s="5" t="s">
         <v>371</v>
       </c>
@@ -10009,17 +10730,20 @@
       <c r="Q84" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="R84" s="10" t="s">
+      <c r="R84" s="85" t="s">
+        <v>1464</v>
+      </c>
+      <c r="S84" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S84" s="80" t="s">
+      <c r="T84" s="80" t="s">
         <v>1300</v>
       </c>
-      <c r="T84" s="82" t="s">
+      <c r="U84" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="85" spans="1:20" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A85" s="5" t="s">
         <v>374</v>
       </c>
@@ -10061,17 +10785,20 @@
       <c r="Q85" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R85" s="10" t="s">
+      <c r="R85" s="85" t="s">
+        <v>1465</v>
+      </c>
+      <c r="S85" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S85" s="80" t="s">
+      <c r="T85" s="80" t="s">
         <v>1304</v>
       </c>
-      <c r="T85" s="82" t="s">
+      <c r="U85" s="82" t="s">
         <v>1322</v>
       </c>
     </row>
-    <row r="86" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A86" s="5" t="s">
         <v>391</v>
       </c>
@@ -10121,17 +10848,20 @@
       <c r="Q86" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="R86" s="10" t="s">
+      <c r="R86" s="85" t="s">
+        <v>1466</v>
+      </c>
+      <c r="S86" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S86" s="80" t="s">
+      <c r="T86" s="80" t="s">
         <v>1302</v>
       </c>
-      <c r="T86" s="82" t="s">
+      <c r="U86" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="87" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A87" s="5" t="s">
         <v>378</v>
       </c>
@@ -10181,17 +10911,20 @@
       <c r="Q87" s="41" t="s">
         <v>266</v>
       </c>
-      <c r="R87" s="10" t="s">
+      <c r="R87" s="85" t="s">
+        <v>1467</v>
+      </c>
+      <c r="S87" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S87" s="80" t="s">
+      <c r="T87" s="80" t="s">
         <v>1302</v>
       </c>
-      <c r="T87" s="82" t="s">
+      <c r="U87" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="88" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A88" s="5" t="s">
         <v>384</v>
       </c>
@@ -10235,17 +10968,20 @@
       <c r="Q88" s="10" t="s">
         <v>389</v>
       </c>
-      <c r="R88" s="10" t="s">
+      <c r="R88" s="85" t="s">
+        <v>1468</v>
+      </c>
+      <c r="S88" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S88" s="80" t="s">
+      <c r="T88" s="80" t="s">
         <v>1302</v>
       </c>
-      <c r="T88" s="82" t="s">
+      <c r="U88" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="89" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A89" s="5" t="s">
         <v>396</v>
       </c>
@@ -10291,17 +11027,20 @@
       <c r="Q89" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="R89" s="10" t="s">
+      <c r="R89" s="85" t="s">
+        <v>1469</v>
+      </c>
+      <c r="S89" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S89" s="80" t="s">
+      <c r="T89" s="80" t="s">
         <v>1305</v>
       </c>
-      <c r="T89" s="82" t="s">
+      <c r="U89" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="90" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A90" s="5" t="s">
         <v>401</v>
       </c>
@@ -10343,17 +11082,20 @@
       <c r="Q90" s="41" t="s">
         <v>404</v>
       </c>
-      <c r="R90" s="10" t="s">
+      <c r="R90" s="85" t="s">
+        <v>1470</v>
+      </c>
+      <c r="S90" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S90" s="80" t="s">
+      <c r="T90" s="80" t="s">
         <v>1305</v>
       </c>
-      <c r="T90" s="82" t="s">
+      <c r="U90" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="91" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A91" s="5" t="s">
         <v>406</v>
       </c>
@@ -10395,17 +11137,20 @@
       <c r="Q91" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="R91" s="10" t="s">
+      <c r="R91" s="85" t="s">
+        <v>1471</v>
+      </c>
+      <c r="S91" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S91" s="80" t="s">
+      <c r="T91" s="80" t="s">
         <v>1305</v>
       </c>
-      <c r="T91" s="82" t="s">
+      <c r="U91" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="92" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A92" s="5" t="s">
         <v>411</v>
       </c>
@@ -10449,17 +11194,20 @@
       <c r="Q92" s="10" t="s">
         <v>413</v>
       </c>
-      <c r="R92" s="10" t="s">
+      <c r="R92" s="85" t="s">
+        <v>1472</v>
+      </c>
+      <c r="S92" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S92" s="80" t="s">
+      <c r="T92" s="80" t="s">
         <v>1305</v>
       </c>
-      <c r="T92" s="82" t="s">
+      <c r="U92" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="93" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A93" s="5" t="s">
         <v>415</v>
       </c>
@@ -10501,17 +11249,20 @@
       <c r="Q93" s="10" t="s">
         <v>389</v>
       </c>
-      <c r="R93" s="10" t="s">
+      <c r="R93" s="85" t="s">
+        <v>1473</v>
+      </c>
+      <c r="S93" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S93" s="80" t="s">
+      <c r="T93" s="80" t="s">
         <v>1305</v>
       </c>
-      <c r="T93" s="82" t="s">
+      <c r="U93" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="94" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A94" s="26" t="s">
         <v>778</v>
       </c>
@@ -10555,17 +11306,20 @@
       <c r="Q94" s="33" t="s">
         <v>389</v>
       </c>
-      <c r="R94" s="5" t="s">
+      <c r="R94" s="85" t="s">
+        <v>1474</v>
+      </c>
+      <c r="S94" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="S94" s="80" t="s">
+      <c r="T94" s="80" t="s">
         <v>1305</v>
       </c>
-      <c r="T94" s="82" t="s">
+      <c r="U94" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="95" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A95" s="5" t="s">
         <v>418</v>
       </c>
@@ -10615,17 +11369,20 @@
       <c r="Q95" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R95" s="10" t="s">
+      <c r="R95" s="85" t="s">
+        <v>1475</v>
+      </c>
+      <c r="S95" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S95" s="80" t="s">
+      <c r="T95" s="80" t="s">
         <v>1309</v>
       </c>
-      <c r="T95" s="82" t="s">
+      <c r="U95" s="82" t="s">
         <v>1323</v>
       </c>
     </row>
-    <row r="96" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A96" s="5" t="s">
         <v>424</v>
       </c>
@@ -10669,17 +11426,20 @@
       <c r="Q96" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="R96" s="10" t="s">
+      <c r="R96" s="85" t="s">
+        <v>1476</v>
+      </c>
+      <c r="S96" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S96" s="80" t="s">
+      <c r="T96" s="80" t="s">
         <v>1306</v>
       </c>
-      <c r="T96" s="82" t="s">
+      <c r="U96" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="97" spans="1:20" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A97" s="5" t="s">
         <v>428</v>
       </c>
@@ -10727,17 +11487,20 @@
       <c r="Q97" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R97" s="10" t="s">
+      <c r="R97" s="85" t="s">
+        <v>1477</v>
+      </c>
+      <c r="S97" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S97" s="80" t="s">
+      <c r="T97" s="80" t="s">
         <v>1306</v>
       </c>
-      <c r="T97" s="82" t="s">
+      <c r="U97" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="98" spans="1:20" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A98" s="5" t="s">
         <v>421</v>
       </c>
@@ -10781,17 +11544,20 @@
       <c r="Q98" s="41" t="s">
         <v>57</v>
       </c>
-      <c r="R98" s="10" t="s">
+      <c r="R98" s="85" t="s">
+        <v>1478</v>
+      </c>
+      <c r="S98" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S98" s="80" t="s">
+      <c r="T98" s="80" t="s">
         <v>1306</v>
       </c>
-      <c r="T98" s="82" t="s">
+      <c r="U98" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="99" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A99" s="5" t="s">
         <v>431</v>
       </c>
@@ -10835,17 +11601,20 @@
       <c r="Q99" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="R99" s="10" t="s">
+      <c r="R99" s="85" t="s">
+        <v>1479</v>
+      </c>
+      <c r="S99" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S99" s="80" t="s">
+      <c r="T99" s="80" t="s">
         <v>1306</v>
       </c>
-      <c r="T99" s="82" t="s">
+      <c r="U99" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="100" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A100" s="5" t="s">
         <v>435</v>
       </c>
@@ -10893,17 +11662,20 @@
       <c r="Q100" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R100" s="10" t="s">
+      <c r="R100" s="85" t="s">
+        <v>1480</v>
+      </c>
+      <c r="S100" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S100" s="80" t="s">
+      <c r="T100" s="80" t="s">
         <v>1306</v>
       </c>
-      <c r="T100" s="82" t="s">
+      <c r="U100" s="82" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="101" spans="1:20" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A101" s="5" t="s">
         <v>438</v>
       </c>
@@ -10945,17 +11717,20 @@
       <c r="Q101" s="41" t="s">
         <v>57</v>
       </c>
-      <c r="R101" s="10" t="s">
+      <c r="R101" s="85" t="s">
+        <v>1481</v>
+      </c>
+      <c r="S101" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="S101" s="80" t="s">
+      <c r="T101" s="80" t="s">
         <v>1307</v>
       </c>
-      <c r="T101" s="82" t="s">
+      <c r="U101" s="82" t="s">
         <v>1322</v>
       </c>
     </row>
-    <row r="102" spans="1:20" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A102" s="5" t="s">
         <v>460</v>
       </c>
@@ -10995,14 +11770,17 @@
       <c r="Q102" s="10" t="s">
         <v>413</v>
       </c>
-      <c r="R102" s="10" t="s">
+      <c r="R102" s="85" t="s">
+        <v>1482</v>
+      </c>
+      <c r="S102" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="S102" s="42" t="s">
+      <c r="T102" s="42" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="103" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A103" s="5" t="s">
         <v>465</v>
       </c>
@@ -11042,14 +11820,17 @@
       <c r="Q103" s="10" t="s">
         <v>197</v>
       </c>
-      <c r="R103" s="10" t="s">
+      <c r="R103" s="85" t="s">
+        <v>1483</v>
+      </c>
+      <c r="S103" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="S103" s="42" t="s">
+      <c r="T103" s="42" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="104" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A104" s="5" t="s">
         <v>469</v>
       </c>
@@ -11089,14 +11870,17 @@
       <c r="Q104" s="10" t="s">
         <v>471</v>
       </c>
-      <c r="R104" s="10" t="s">
+      <c r="R104" s="85" t="s">
+        <v>1484</v>
+      </c>
+      <c r="S104" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="S104" s="42" t="s">
+      <c r="T104" s="42" t="s">
         <v>472</v>
       </c>
     </row>
-    <row r="105" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A105" s="5" t="s">
         <v>474</v>
       </c>
@@ -11136,14 +11920,17 @@
       <c r="Q105" s="10" t="s">
         <v>389</v>
       </c>
-      <c r="R105" s="10" t="s">
+      <c r="R105" s="85" t="s">
+        <v>1485</v>
+      </c>
+      <c r="S105" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="S105" s="42" t="s">
+      <c r="T105" s="42" t="s">
         <v>476</v>
       </c>
     </row>
-    <row r="106" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A106" s="26" t="s">
         <v>784</v>
       </c>
@@ -11175,9 +11962,12 @@
       <c r="O106" s="41"/>
       <c r="P106" s="37"/>
       <c r="Q106" s="42"/>
-      <c r="R106" s="4"/>
-    </row>
-    <row r="107" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+      <c r="R106" s="85" t="s">
+        <v>1486</v>
+      </c>
+      <c r="S106" s="4"/>
+    </row>
+    <row r="107" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A107" s="5" t="s">
         <v>478</v>
       </c>
@@ -11215,14 +12005,17 @@
       <c r="Q107" s="41" t="s">
         <v>413</v>
       </c>
-      <c r="R107" s="10" t="s">
+      <c r="R107" s="85" t="s">
+        <v>1487</v>
+      </c>
+      <c r="S107" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="S107" s="42" t="s">
+      <c r="T107" s="42" t="s">
         <v>481</v>
       </c>
     </row>
-    <row r="108" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A108" s="5" t="s">
         <v>483</v>
       </c>
@@ -11264,14 +12057,17 @@
       <c r="Q108" s="41" t="s">
         <v>485</v>
       </c>
-      <c r="R108" s="10" t="s">
+      <c r="R108" s="85" t="s">
+        <v>1488</v>
+      </c>
+      <c r="S108" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="S108" s="42" t="s">
+      <c r="T108" s="42" t="s">
         <v>472</v>
       </c>
     </row>
-    <row r="109" spans="1:20" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A109" s="5" t="s">
         <v>487</v>
       </c>
@@ -11313,14 +12109,17 @@
       <c r="Q109" s="41" t="s">
         <v>489</v>
       </c>
-      <c r="R109" s="10" t="s">
+      <c r="R109" s="85" t="s">
+        <v>1489</v>
+      </c>
+      <c r="S109" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="S109" s="42" t="s">
+      <c r="T109" s="42" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="110" spans="1:20" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A110" s="5" t="s">
         <v>492</v>
       </c>
@@ -11360,14 +12159,17 @@
       <c r="Q110" s="41" t="s">
         <v>494</v>
       </c>
-      <c r="R110" s="10" t="s">
+      <c r="R110" s="85" t="s">
+        <v>1490</v>
+      </c>
+      <c r="S110" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="S110" s="42" t="s">
+      <c r="T110" s="42" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="111" spans="1:20" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A111" s="5" t="s">
         <v>496</v>
       </c>
@@ -11407,14 +12209,17 @@
       <c r="Q111" s="41" t="s">
         <v>498</v>
       </c>
-      <c r="R111" s="10" t="s">
+      <c r="R111" s="85" t="s">
+        <v>1491</v>
+      </c>
+      <c r="S111" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="S111" s="42" t="s">
+      <c r="T111" s="42" t="s">
         <v>472</v>
       </c>
     </row>
-    <row r="112" spans="1:20" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A112" s="5" t="s">
         <v>500</v>
       </c>
@@ -11458,14 +12263,17 @@
       <c r="Q112" s="10" t="s">
         <v>504</v>
       </c>
-      <c r="R112" s="10" t="s">
+      <c r="R112" s="85" t="s">
+        <v>1492</v>
+      </c>
+      <c r="S112" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="S112" s="42" t="s">
+      <c r="T112" s="42" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="113" spans="1:23" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:24" ht="72" x14ac:dyDescent="0.3">
       <c r="A113" s="5" t="s">
         <v>506</v>
       </c>
@@ -11513,14 +12321,17 @@
       <c r="Q113" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="R113" s="10" t="s">
+      <c r="R113" s="85" t="s">
+        <v>1493</v>
+      </c>
+      <c r="S113" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="S113" s="42" t="s">
+      <c r="T113" s="42" t="s">
         <v>472</v>
       </c>
     </row>
-    <row r="114" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A114" s="5" t="s">
         <v>511</v>
       </c>
@@ -11566,14 +12377,17 @@
         <v>111</v>
       </c>
       <c r="Q114" s="41"/>
-      <c r="R114" s="10" t="s">
+      <c r="R114" s="85" t="s">
+        <v>111</v>
+      </c>
+      <c r="S114" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="S114" s="42" t="s">
+      <c r="T114" s="42" t="s">
         <v>512</v>
       </c>
     </row>
-    <row r="115" spans="1:23" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A115" s="5" t="s">
         <v>443</v>
       </c>
@@ -11615,14 +12429,17 @@
       <c r="Q115" s="41" t="s">
         <v>447</v>
       </c>
-      <c r="R115" s="10" t="s">
+      <c r="R115" s="85" t="s">
+        <v>1494</v>
+      </c>
+      <c r="S115" s="10" t="s">
         <v>1378</v>
       </c>
-      <c r="S115" s="4" t="s">
+      <c r="T115" s="4" t="s">
         <v>1379</v>
       </c>
     </row>
-    <row r="116" spans="1:23" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A116" s="5" t="s">
         <v>450</v>
       </c>
@@ -11670,14 +12487,17 @@
       <c r="Q116" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R116" s="10" t="s">
+      <c r="R116" s="85" t="s">
+        <v>1495</v>
+      </c>
+      <c r="S116" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="S116" s="42" t="s">
+      <c r="T116" s="42" t="s">
         <v>452</v>
       </c>
     </row>
-    <row r="117" spans="1:23" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:24" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A117" s="5" t="s">
         <v>454</v>
       </c>
@@ -11717,14 +12537,17 @@
       <c r="Q117" s="41" t="s">
         <v>457</v>
       </c>
-      <c r="R117" s="10" t="s">
+      <c r="R117" s="85" t="s">
+        <v>1496</v>
+      </c>
+      <c r="S117" s="10" t="s">
         <v>448</v>
       </c>
-      <c r="S117" s="42" t="s">
+      <c r="T117" s="42" t="s">
         <v>458</v>
       </c>
     </row>
-    <row r="118" spans="1:23" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A118" s="5" t="s">
         <v>514</v>
       </c>
@@ -11766,14 +12589,17 @@
       <c r="Q118" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="R118" s="10" t="s">
+      <c r="R118" s="85" t="s">
+        <v>1497</v>
+      </c>
+      <c r="S118" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S118" s="43" t="s">
+      <c r="T118" s="43" t="s">
         <v>1362</v>
       </c>
     </row>
-    <row r="119" spans="1:23" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A119" s="5" t="s">
         <v>521</v>
       </c>
@@ -11817,14 +12643,17 @@
       <c r="Q119" s="41" t="s">
         <v>523</v>
       </c>
-      <c r="R119" s="10" t="s">
+      <c r="R119" s="85" t="s">
+        <v>1498</v>
+      </c>
+      <c r="S119" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S119" s="43" t="s">
+      <c r="T119" s="43" t="s">
         <v>1362</v>
       </c>
     </row>
-    <row r="120" spans="1:23" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:24" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A120" s="26" t="s">
         <v>785</v>
       </c>
@@ -11868,14 +12697,17 @@
       <c r="Q120" s="33" t="s">
         <v>788</v>
       </c>
-      <c r="R120" s="5" t="s">
+      <c r="R120" s="85" t="s">
+        <v>1499</v>
+      </c>
+      <c r="S120" s="5" t="s">
         <v>519</v>
       </c>
-      <c r="S120" s="43" t="s">
+      <c r="T120" s="43" t="s">
         <v>1363</v>
       </c>
     </row>
-    <row r="121" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A121" s="5" t="s">
         <v>525</v>
       </c>
@@ -11919,14 +12751,17 @@
       <c r="Q121" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="R121" s="10" t="s">
+      <c r="R121" s="85" t="s">
+        <v>1500</v>
+      </c>
+      <c r="S121" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S121" s="4" t="s">
+      <c r="T121" s="4" t="s">
         <v>1364</v>
       </c>
     </row>
-    <row r="122" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A122" s="5" t="s">
         <v>529</v>
       </c>
@@ -11970,14 +12805,17 @@
       <c r="Q122" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="R122" s="10" t="s">
+      <c r="R122" s="85" t="s">
+        <v>1501</v>
+      </c>
+      <c r="S122" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S122" s="4" t="s">
+      <c r="T122" s="4" t="s">
         <v>1365</v>
       </c>
     </row>
-    <row r="123" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A123" s="5" t="s">
         <v>532</v>
       </c>
@@ -12019,14 +12857,17 @@
       <c r="Q123" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="R123" s="10" t="s">
+      <c r="R123" s="85" t="s">
+        <v>1502</v>
+      </c>
+      <c r="S123" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S123" s="4" t="s">
+      <c r="T123" s="4" t="s">
         <v>1364</v>
       </c>
     </row>
-    <row r="124" spans="1:23" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:24" ht="72" x14ac:dyDescent="0.3">
       <c r="A124" s="5" t="s">
         <v>535</v>
       </c>
@@ -12076,14 +12917,17 @@
       <c r="Q124" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R124" s="10" t="s">
+      <c r="R124" s="85" t="s">
+        <v>1503</v>
+      </c>
+      <c r="S124" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S124" s="43" t="s">
+      <c r="T124" s="43" t="s">
         <v>1362</v>
       </c>
     </row>
-    <row r="125" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A125" s="5" t="s">
         <v>540</v>
       </c>
@@ -12131,15 +12975,18 @@
       <c r="Q125" s="10" t="s">
         <v>485</v>
       </c>
-      <c r="R125" s="10" t="s">
+      <c r="R125" s="85" t="s">
+        <v>1502</v>
+      </c>
+      <c r="S125" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S125" s="4" t="s">
+      <c r="T125" s="4" t="s">
         <v>1366</v>
       </c>
-      <c r="W125" s="4"/>
-    </row>
-    <row r="126" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X125" s="4"/>
+    </row>
+    <row r="126" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A126" s="26" t="s">
         <v>795</v>
       </c>
@@ -12187,15 +13034,18 @@
       <c r="Q126" s="79" t="s">
         <v>66</v>
       </c>
-      <c r="R126" s="5" t="s">
+      <c r="R126" s="85" t="s">
+        <v>1504</v>
+      </c>
+      <c r="S126" s="5" t="s">
         <v>519</v>
       </c>
-      <c r="S126" s="43" t="s">
+      <c r="T126" s="43" t="s">
         <v>1367</v>
       </c>
-      <c r="W126" s="4"/>
-    </row>
-    <row r="127" spans="1:23" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="X126" s="4"/>
+    </row>
+    <row r="127" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A127" s="5" t="s">
         <v>546</v>
       </c>
@@ -12245,15 +13095,18 @@
       <c r="Q127" s="38" t="s">
         <v>100</v>
       </c>
-      <c r="R127" s="10" t="s">
+      <c r="R127" s="85" t="s">
+        <v>1505</v>
+      </c>
+      <c r="S127" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S127" s="43" t="s">
+      <c r="T127" s="43" t="s">
         <v>1362</v>
       </c>
-      <c r="W127" s="4"/>
-    </row>
-    <row r="128" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X127" s="4"/>
+    </row>
+    <row r="128" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A128" s="5" t="s">
         <v>549</v>
       </c>
@@ -12305,15 +13158,18 @@
       <c r="Q128" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="R128" s="10" t="s">
+      <c r="R128" s="85" t="s">
+        <v>1506</v>
+      </c>
+      <c r="S128" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S128" s="4" t="s">
+      <c r="T128" s="4" t="s">
         <v>1364</v>
       </c>
-      <c r="W128" s="4"/>
-    </row>
-    <row r="129" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X128" s="4"/>
+    </row>
+    <row r="129" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A129" s="5" t="s">
         <v>554</v>
       </c>
@@ -12363,15 +13219,18 @@
       <c r="Q129" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="R129" s="10" t="s">
+      <c r="R129" s="85" t="s">
+        <v>1507</v>
+      </c>
+      <c r="S129" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S129" s="4" t="s">
+      <c r="T129" s="4" t="s">
         <v>1364</v>
       </c>
-      <c r="W129" s="4"/>
-    </row>
-    <row r="130" spans="1:23" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="X129" s="4"/>
+    </row>
+    <row r="130" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A130" s="26" t="s">
         <v>798</v>
       </c>
@@ -12419,15 +13278,18 @@
       <c r="Q130" s="24" t="s">
         <v>266</v>
       </c>
-      <c r="R130" s="5" t="s">
+      <c r="R130" s="85" t="s">
+        <v>1508</v>
+      </c>
+      <c r="S130" s="5" t="s">
         <v>519</v>
       </c>
-      <c r="S130" s="4" t="s">
+      <c r="T130" s="4" t="s">
         <v>1368</v>
       </c>
-      <c r="W130" s="4"/>
-    </row>
-    <row r="131" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X130" s="4"/>
+    </row>
+    <row r="131" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A131" s="26" t="s">
         <v>802</v>
       </c>
@@ -12475,15 +13337,18 @@
       <c r="Q131" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="R131" s="5" t="s">
+      <c r="R131" s="85" t="s">
+        <v>1509</v>
+      </c>
+      <c r="S131" s="5" t="s">
         <v>519</v>
       </c>
-      <c r="S131" s="4" t="s">
+      <c r="T131" s="4" t="s">
         <v>1369</v>
       </c>
-      <c r="W131" s="4"/>
-    </row>
-    <row r="132" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X131" s="4"/>
+    </row>
+    <row r="132" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A132" s="5" t="s">
         <v>558</v>
       </c>
@@ -12531,15 +13396,18 @@
       <c r="Q132" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="R132" s="10" t="s">
+      <c r="R132" s="85" t="s">
+        <v>1510</v>
+      </c>
+      <c r="S132" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S132" s="43" t="s">
+      <c r="T132" s="43" t="s">
         <v>1362</v>
       </c>
-      <c r="W132" s="4"/>
-    </row>
-    <row r="133" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X132" s="4"/>
+    </row>
+    <row r="133" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A133" s="5" t="s">
         <v>561</v>
       </c>
@@ -12589,15 +13457,18 @@
       <c r="Q133" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="R133" s="10" t="s">
+      <c r="R133" s="85" t="s">
+        <v>1511</v>
+      </c>
+      <c r="S133" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S133" s="43" t="s">
+      <c r="T133" s="43" t="s">
         <v>1362</v>
       </c>
-      <c r="W133" s="4"/>
-    </row>
-    <row r="134" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X133" s="4"/>
+    </row>
+    <row r="134" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A134" s="5" t="s">
         <v>564</v>
       </c>
@@ -12645,15 +13516,18 @@
       <c r="Q134" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="R134" s="10" t="s">
+      <c r="R134" s="85" t="s">
+        <v>1512</v>
+      </c>
+      <c r="S134" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S134" s="4" t="s">
+      <c r="T134" s="4" t="s">
         <v>1370</v>
       </c>
-      <c r="W134" s="4"/>
-    </row>
-    <row r="135" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X134" s="4"/>
+    </row>
+    <row r="135" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A135" s="5" t="s">
         <v>568</v>
       </c>
@@ -12703,15 +13577,18 @@
       <c r="Q135" s="41" t="s">
         <v>159</v>
       </c>
-      <c r="R135" s="10" t="s">
+      <c r="R135" s="85" t="s">
+        <v>1513</v>
+      </c>
+      <c r="S135" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S135" s="4" t="s">
+      <c r="T135" s="4" t="s">
         <v>1364</v>
       </c>
-      <c r="W135" s="4"/>
-    </row>
-    <row r="136" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X135" s="4"/>
+    </row>
+    <row r="136" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A136" s="5" t="s">
         <v>571</v>
       </c>
@@ -12759,15 +13636,18 @@
       <c r="Q136" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="R136" s="10" t="s">
+      <c r="R136" s="85" t="s">
+        <v>1514</v>
+      </c>
+      <c r="S136" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S136" s="4" t="s">
+      <c r="T136" s="4" t="s">
         <v>1364</v>
       </c>
-      <c r="W136" s="4"/>
-    </row>
-    <row r="137" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X136" s="4"/>
+    </row>
+    <row r="137" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A137" s="5" t="s">
         <v>574</v>
       </c>
@@ -12819,15 +13699,18 @@
       <c r="Q137" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="R137" s="10" t="s">
+      <c r="R137" s="85" t="s">
+        <v>1515</v>
+      </c>
+      <c r="S137" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S137" s="4" t="s">
+      <c r="T137" s="4" t="s">
         <v>1364</v>
       </c>
-      <c r="W137" s="4"/>
-    </row>
-    <row r="138" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X137" s="4"/>
+    </row>
+    <row r="138" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A138" s="26" t="s">
         <v>805</v>
       </c>
@@ -12877,15 +13760,18 @@
       <c r="Q138" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="R138" s="5" t="s">
+      <c r="R138" s="85" t="s">
+        <v>1516</v>
+      </c>
+      <c r="S138" s="5" t="s">
         <v>519</v>
       </c>
-      <c r="S138" s="43" t="s">
+      <c r="T138" s="43" t="s">
         <v>1371</v>
       </c>
-      <c r="W138" s="4"/>
-    </row>
-    <row r="139" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X138" s="4"/>
+    </row>
+    <row r="139" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A139" s="26" t="s">
         <v>808</v>
       </c>
@@ -12933,15 +13819,18 @@
       <c r="Q139" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="R139" s="5" t="s">
+      <c r="R139" s="85" t="s">
+        <v>1517</v>
+      </c>
+      <c r="S139" s="5" t="s">
         <v>519</v>
       </c>
-      <c r="S139" s="4" t="s">
+      <c r="T139" s="4" t="s">
         <v>1364</v>
       </c>
-      <c r="W139" s="4"/>
-    </row>
-    <row r="140" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X139" s="4"/>
+    </row>
+    <row r="140" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A140" s="5" t="s">
         <v>579</v>
       </c>
@@ -12991,15 +13880,18 @@
       <c r="Q140" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="R140" s="10" t="s">
+      <c r="R140" s="85" t="s">
+        <v>1518</v>
+      </c>
+      <c r="S140" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S140" s="4" t="s">
+      <c r="T140" s="4" t="s">
         <v>1372</v>
       </c>
-      <c r="W140" s="4"/>
-    </row>
-    <row r="141" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X140" s="4"/>
+    </row>
+    <row r="141" spans="1:24" ht="72" x14ac:dyDescent="0.3">
       <c r="A141" s="5" t="s">
         <v>582</v>
       </c>
@@ -13049,15 +13941,18 @@
       <c r="Q141" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R141" s="10" t="s">
+      <c r="R141" s="85" t="s">
+        <v>1519</v>
+      </c>
+      <c r="S141" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S141" s="4" t="s">
+      <c r="T141" s="4" t="s">
         <v>1373</v>
       </c>
-      <c r="W141" s="4"/>
-    </row>
-    <row r="142" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X141" s="4"/>
+    </row>
+    <row r="142" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A142" s="5" t="s">
         <v>586</v>
       </c>
@@ -13107,15 +14002,18 @@
       <c r="Q142" s="10" t="s">
         <v>588</v>
       </c>
-      <c r="R142" s="10" t="s">
+      <c r="R142" s="85" t="s">
+        <v>1520</v>
+      </c>
+      <c r="S142" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S142" s="43" t="s">
+      <c r="T142" s="43" t="s">
         <v>1374</v>
       </c>
-      <c r="W142" s="4"/>
-    </row>
-    <row r="143" spans="1:23" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="X142" s="4"/>
+    </row>
+    <row r="143" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A143" s="5" t="s">
         <v>590</v>
       </c>
@@ -13163,15 +14061,18 @@
       <c r="Q143" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R143" s="10" t="s">
+      <c r="R143" s="85" t="s">
+        <v>1521</v>
+      </c>
+      <c r="S143" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S143" s="4" t="s">
+      <c r="T143" s="4" t="s">
         <v>1375</v>
       </c>
-      <c r="W143" s="4"/>
-    </row>
-    <row r="144" spans="1:23" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="X143" s="4"/>
+    </row>
+    <row r="144" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A144" s="5" t="s">
         <v>595</v>
       </c>
@@ -13221,15 +14122,18 @@
       <c r="Q144" s="10" t="s">
         <v>598</v>
       </c>
-      <c r="R144" s="10" t="s">
+      <c r="R144" s="85" t="s">
+        <v>1522</v>
+      </c>
+      <c r="S144" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S144" s="4" t="s">
+      <c r="T144" s="4" t="s">
         <v>1368</v>
       </c>
-      <c r="W144" s="4"/>
-    </row>
-    <row r="145" spans="1:23" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="X144" s="4"/>
+    </row>
+    <row r="145" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A145" s="26" t="s">
         <v>811</v>
       </c>
@@ -13277,15 +14181,18 @@
       <c r="Q145" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="R145" s="5" t="s">
+      <c r="R145" s="85" t="s">
+        <v>1523</v>
+      </c>
+      <c r="S145" s="5" t="s">
         <v>519</v>
       </c>
-      <c r="S145" s="43" t="s">
+      <c r="T145" s="43" t="s">
         <v>1376</v>
       </c>
-      <c r="W145" s="4"/>
-    </row>
-    <row r="146" spans="1:23" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="X145" s="4"/>
+    </row>
+    <row r="146" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A146" s="5" t="s">
         <v>600</v>
       </c>
@@ -13335,15 +14242,18 @@
       <c r="Q146" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="R146" s="10" t="s">
+      <c r="R146" s="85" t="s">
+        <v>1524</v>
+      </c>
+      <c r="S146" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S146" s="43" t="s">
+      <c r="T146" s="43" t="s">
         <v>1374</v>
       </c>
-      <c r="W146" s="4"/>
-    </row>
-    <row r="147" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X146" s="4"/>
+    </row>
+    <row r="147" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A147" s="26" t="s">
         <v>815</v>
       </c>
@@ -13393,15 +14303,18 @@
       <c r="Q147" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="R147" s="5" t="s">
+      <c r="R147" s="85" t="s">
+        <v>1525</v>
+      </c>
+      <c r="S147" s="5" t="s">
         <v>519</v>
       </c>
-      <c r="S147" s="43" t="s">
+      <c r="T147" s="43" t="s">
         <v>1374</v>
       </c>
-      <c r="W147" s="4"/>
-    </row>
-    <row r="148" spans="1:23" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="X147" s="4"/>
+    </row>
+    <row r="148" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A148" s="5" t="s">
         <v>605</v>
       </c>
@@ -13449,15 +14362,18 @@
       <c r="Q148" s="10" t="s">
         <v>211</v>
       </c>
-      <c r="R148" s="10" t="s">
+      <c r="R148" s="85" t="s">
+        <v>1526</v>
+      </c>
+      <c r="S148" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S148" s="43" t="s">
+      <c r="T148" s="43" t="s">
         <v>1374</v>
       </c>
-      <c r="W148" s="4"/>
-    </row>
-    <row r="149" spans="1:23" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="X148" s="4"/>
+    </row>
+    <row r="149" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A149" s="5" t="s">
         <v>610</v>
       </c>
@@ -13505,15 +14421,18 @@
       <c r="Q149" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="R149" s="10" t="s">
+      <c r="R149" s="85" t="s">
+        <v>1527</v>
+      </c>
+      <c r="S149" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S149" s="4" t="s">
+      <c r="T149" s="4" t="s">
         <v>1366</v>
       </c>
-      <c r="W149" s="4"/>
-    </row>
-    <row r="150" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X149" s="4"/>
+    </row>
+    <row r="150" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A150" s="5" t="s">
         <v>615</v>
       </c>
@@ -13561,15 +14480,18 @@
       <c r="Q150" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="R150" s="10" t="s">
+      <c r="R150" s="85" t="s">
+        <v>1528</v>
+      </c>
+      <c r="S150" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S150" s="4" t="s">
+      <c r="T150" s="4" t="s">
         <v>1364</v>
       </c>
-      <c r="W150" s="4"/>
-    </row>
-    <row r="151" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X150" s="4"/>
+    </row>
+    <row r="151" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A151" s="5" t="s">
         <v>618</v>
       </c>
@@ -13619,15 +14541,18 @@
       <c r="Q151" s="41" t="s">
         <v>622</v>
       </c>
-      <c r="R151" s="10" t="s">
+      <c r="R151" s="85" t="s">
+        <v>1529</v>
+      </c>
+      <c r="S151" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S151" s="4" t="s">
+      <c r="T151" s="4" t="s">
         <v>1368</v>
       </c>
-      <c r="W151" s="4"/>
-    </row>
-    <row r="152" spans="1:23" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="X151" s="4"/>
+    </row>
+    <row r="152" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A152" s="26" t="s">
         <v>817</v>
       </c>
@@ -13675,15 +14600,18 @@
       <c r="Q152" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="R152" s="5" t="s">
+      <c r="R152" s="85" t="s">
+        <v>1530</v>
+      </c>
+      <c r="S152" s="5" t="s">
         <v>519</v>
       </c>
-      <c r="S152" s="4" t="s">
+      <c r="T152" s="4" t="s">
         <v>1364</v>
       </c>
-      <c r="W152" s="4"/>
-    </row>
-    <row r="153" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X152" s="4"/>
+    </row>
+    <row r="153" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A153" s="5" t="s">
         <v>624</v>
       </c>
@@ -13731,15 +14659,18 @@
       <c r="Q153" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="R153" s="10" t="s">
+      <c r="R153" s="85" t="s">
+        <v>1531</v>
+      </c>
+      <c r="S153" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S153" s="4" t="s">
+      <c r="T153" s="4" t="s">
         <v>1368</v>
       </c>
-      <c r="W153" s="4"/>
-    </row>
-    <row r="154" spans="1:23" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="X153" s="4"/>
+    </row>
+    <row r="154" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A154" s="5" t="s">
         <v>628</v>
       </c>
@@ -13787,15 +14718,18 @@
       <c r="Q154" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="R154" s="10" t="s">
+      <c r="R154" s="85" t="s">
+        <v>1532</v>
+      </c>
+      <c r="S154" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S154" s="4" t="s">
+      <c r="T154" s="4" t="s">
         <v>1373</v>
       </c>
-      <c r="W154" s="4"/>
-    </row>
-    <row r="155" spans="1:23" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="X154" s="4"/>
+    </row>
+    <row r="155" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A155" s="26" t="s">
         <v>819</v>
       </c>
@@ -13843,15 +14777,18 @@
       <c r="Q155" s="33" t="s">
         <v>821</v>
       </c>
-      <c r="R155" s="5" t="s">
+      <c r="R155" s="85" t="s">
+        <v>1533</v>
+      </c>
+      <c r="S155" s="5" t="s">
         <v>519</v>
       </c>
-      <c r="S155" s="43" t="s">
+      <c r="T155" s="43" t="s">
         <v>1377</v>
       </c>
-      <c r="W155" s="4"/>
-    </row>
-    <row r="156" spans="1:23" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="X155" s="4"/>
+    </row>
+    <row r="156" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A156" s="5" t="s">
         <v>632</v>
       </c>
@@ -13899,15 +14836,18 @@
       <c r="Q156" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="R156" s="10" t="s">
+      <c r="R156" s="85" t="s">
+        <v>1534</v>
+      </c>
+      <c r="S156" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S156" s="4" t="s">
+      <c r="T156" s="4" t="s">
         <v>1369</v>
       </c>
-      <c r="W156" s="4"/>
-    </row>
-    <row r="157" spans="1:23" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="X156" s="4"/>
+    </row>
+    <row r="157" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A157" s="5" t="s">
         <v>635</v>
       </c>
@@ -13957,15 +14897,18 @@
       <c r="Q157" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="R157" s="10" t="s">
+      <c r="R157" s="85" t="s">
+        <v>1535</v>
+      </c>
+      <c r="S157" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S157" s="4" t="s">
+      <c r="T157" s="4" t="s">
         <v>1380</v>
       </c>
-      <c r="W157" s="4"/>
-    </row>
-    <row r="158" spans="1:23" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="X157" s="4"/>
+    </row>
+    <row r="158" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A158" s="5" t="s">
         <v>638</v>
       </c>
@@ -14013,15 +14956,16 @@
         <v>641</v>
       </c>
       <c r="Q158" s="41"/>
-      <c r="R158" s="10" t="s">
+      <c r="R158" s="41"/>
+      <c r="S158" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S158" s="42" t="s">
+      <c r="T158" s="42" t="s">
         <v>642</v>
       </c>
-      <c r="W158" s="4"/>
-    </row>
-    <row r="159" spans="1:23" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="X158" s="4"/>
+    </row>
+    <row r="159" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A159" s="5" t="s">
         <v>644</v>
       </c>
@@ -14067,15 +15011,16 @@
         <v>645</v>
       </c>
       <c r="Q159" s="41"/>
-      <c r="R159" s="10" t="s">
+      <c r="R159" s="41"/>
+      <c r="S159" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S159" s="42" t="s">
+      <c r="T159" s="42" t="s">
         <v>642</v>
       </c>
-      <c r="W159" s="4"/>
-    </row>
-    <row r="160" spans="1:23" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="X159" s="4"/>
+    </row>
+    <row r="160" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A160" s="5" t="s">
         <v>647</v>
       </c>
@@ -14123,15 +15068,16 @@
         <v>649</v>
       </c>
       <c r="Q160" s="38"/>
-      <c r="R160" s="10" t="s">
+      <c r="R160" s="41"/>
+      <c r="S160" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S160" s="42" t="s">
+      <c r="T160" s="42" t="s">
         <v>642</v>
       </c>
-      <c r="W160" s="4"/>
-    </row>
-    <row r="161" spans="1:23" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="X160" s="4"/>
+    </row>
+    <row r="161" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A161" s="5" t="s">
         <v>651</v>
       </c>
@@ -14179,15 +15125,16 @@
         <v>652</v>
       </c>
       <c r="Q161" s="38"/>
-      <c r="R161" s="10" t="s">
+      <c r="R161" s="41"/>
+      <c r="S161" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S161" s="42" t="s">
+      <c r="T161" s="42" t="s">
         <v>642</v>
       </c>
-      <c r="W161" s="4"/>
-    </row>
-    <row r="162" spans="1:23" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="X161" s="4"/>
+    </row>
+    <row r="162" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A162" s="5" t="s">
         <v>654</v>
       </c>
@@ -14233,15 +15180,16 @@
         <v>656</v>
       </c>
       <c r="Q162" s="38"/>
-      <c r="R162" s="10" t="s">
+      <c r="R162" s="41"/>
+      <c r="S162" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S162" s="42" t="s">
+      <c r="T162" s="42" t="s">
         <v>642</v>
       </c>
-      <c r="W162" s="4"/>
-    </row>
-    <row r="163" spans="1:23" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="X162" s="4"/>
+    </row>
+    <row r="163" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A163" s="5" t="s">
         <v>658</v>
       </c>
@@ -14287,15 +15235,16 @@
         <v>659</v>
       </c>
       <c r="Q163" s="38"/>
-      <c r="R163" s="10" t="s">
+      <c r="R163" s="41"/>
+      <c r="S163" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S163" s="42" t="s">
+      <c r="T163" s="42" t="s">
         <v>642</v>
       </c>
-      <c r="W163" s="4"/>
-    </row>
-    <row r="164" spans="1:23" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="X163" s="4"/>
+    </row>
+    <row r="164" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A164" s="5" t="s">
         <v>661</v>
       </c>
@@ -14343,15 +15292,16 @@
         <v>663</v>
       </c>
       <c r="Q164" s="38"/>
-      <c r="R164" s="10" t="s">
+      <c r="R164" s="41"/>
+      <c r="S164" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S164" s="42" t="s">
+      <c r="T164" s="42" t="s">
         <v>642</v>
       </c>
-      <c r="W164" s="4"/>
-    </row>
-    <row r="165" spans="1:23" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="X164" s="4"/>
+    </row>
+    <row r="165" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A165" s="5" t="s">
         <v>665</v>
       </c>
@@ -14397,15 +15347,16 @@
         <v>666</v>
       </c>
       <c r="Q165" s="38"/>
-      <c r="R165" s="10" t="s">
+      <c r="R165" s="41"/>
+      <c r="S165" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S165" s="42" t="s">
+      <c r="T165" s="42" t="s">
         <v>642</v>
       </c>
-      <c r="W165" s="4"/>
-    </row>
-    <row r="166" spans="1:23" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
+      <c r="X165" s="4"/>
+    </row>
+    <row r="166" spans="1:24" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A166" s="5" t="s">
         <v>668</v>
       </c>
@@ -14451,15 +15402,16 @@
         <v>669</v>
       </c>
       <c r="Q166" s="38"/>
-      <c r="R166" s="10" t="s">
+      <c r="R166" s="41"/>
+      <c r="S166" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S166" s="42" t="s">
+      <c r="T166" s="42" t="s">
         <v>642</v>
       </c>
-      <c r="W166" s="4"/>
-    </row>
-    <row r="167" spans="1:23" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="X166" s="4"/>
+    </row>
+    <row r="167" spans="1:24" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A167" s="5" t="s">
         <v>671</v>
       </c>
@@ -14503,23 +15455,18 @@
         <v>673</v>
       </c>
       <c r="Q167" s="38"/>
-      <c r="R167" s="10" t="s">
+      <c r="R167" s="41"/>
+      <c r="S167" s="10" t="s">
         <v>519</v>
       </c>
-      <c r="S167" s="42" t="s">
+      <c r="T167" s="42" t="s">
         <v>642</v>
       </c>
-      <c r="W167" s="4"/>
+      <c r="X167" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S167" xr:uid="{647BE94F-31AC-4288-9847-0E65BAB2173D}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="Tashkent"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T167">
+  <autoFilter ref="A1:T167" xr:uid="{647BE94F-31AC-4288-9847-0E65BAB2173D}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:U167">
     <sortCondition ref="A1:A167"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>